<commit_message>
Refactor API components and enhance subscription management: Update ApiPlugin and ApiRequestExecutor for improved caching and error handling, modify GoogleAnalyticsProvider for better script loading, and refine PremiumFeatureBanner and SubscriptionService for enhanced user experience and error management.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\work-time-tracker\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09F32D22-F5A6-44FD-81FA-90E5497223C3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1535" uniqueCount="913">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1536" uniqueCount="914">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5330,6 +5330,10 @@
   </si>
   <si>
     <t>Found 119 errors in 27 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 101 errors in 26 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6102,7 +6106,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D17"/>
+  <dimension ref="B2:D18"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6195,6 +6199,11 @@
     <row r="17" spans="3:3">
       <c r="C17" t="s">
         <v>912</v>
+      </c>
+    </row>
+    <row r="18" spans="3:3">
+      <c r="C18" t="s">
+        <v>913</v>
       </c>
     </row>
   </sheetData>
@@ -6361,7 +6370,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6372,7 +6381,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>00:59</v>
+        <v>01:04</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6571,7 +6580,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6650,7 +6659,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6729,7 +6738,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6808,7 +6817,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -6887,7 +6896,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -6966,7 +6975,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7045,7 +7054,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7124,7 +7133,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7203,7 +7212,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7282,7 +7291,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7361,7 +7370,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7440,7 +7449,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7519,7 +7528,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7598,7 +7607,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7677,7 +7686,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7756,7 +7765,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7835,7 +7844,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -7914,7 +7923,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -7993,7 +8002,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8072,7 +8081,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8151,7 +8160,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8230,7 +8239,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8309,7 +8318,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8388,7 +8397,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8467,7 +8476,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8548,7 +8557,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8629,7 +8638,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8710,7 +8719,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8789,7 +8798,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -8868,7 +8877,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -8947,7 +8956,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9028,7 +9037,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9109,7 +9118,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9190,7 +9199,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9269,7 +9278,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9348,7 +9357,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9427,7 +9436,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9506,7 +9515,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9585,7 +9594,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9666,7 +9675,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9747,7 +9756,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9826,7 +9835,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -9905,7 +9914,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -9984,7 +9993,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10063,7 +10072,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10142,7 +10151,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10223,7 +10232,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10304,7 +10313,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10383,7 +10392,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10462,7 +10471,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10541,7 +10550,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10620,7 +10629,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10699,7 +10708,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10780,7 +10789,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10859,7 +10868,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -10940,7 +10949,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11019,7 +11028,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11098,7 +11107,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11177,7 +11186,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11256,7 +11265,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11335,7 +11344,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11416,7 +11425,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11495,7 +11504,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11574,7 +11583,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11656,7 +11665,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11735,7 +11744,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11814,7 +11823,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -11893,7 +11902,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -11972,7 +11981,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12051,7 +12060,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12130,7 +12139,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12209,7 +12218,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12288,7 +12297,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12367,7 +12376,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12446,7 +12455,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12525,7 +12534,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12604,7 +12613,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12683,7 +12692,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12762,7 +12771,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12841,7 +12850,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -12920,7 +12929,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -12999,7 +13008,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13078,7 +13087,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13157,7 +13166,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13236,7 +13245,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13315,7 +13324,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13394,7 +13403,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13473,7 +13482,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13552,7 +13561,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13631,7 +13640,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13710,7 +13719,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13789,7 +13798,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -13868,7 +13877,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -13947,7 +13956,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14026,7 +14035,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14105,7 +14114,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14184,7 +14193,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14265,7 +14274,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14344,7 +14353,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14423,7 +14432,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14502,7 +14511,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14581,7 +14590,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14660,7 +14669,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14741,7 +14750,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14822,7 +14831,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -14901,7 +14910,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -14980,7 +14989,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15059,7 +15068,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15138,7 +15147,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15219,7 +15228,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15298,7 +15307,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15377,7 +15386,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15456,7 +15465,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15535,7 +15544,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15614,7 +15623,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15693,7 +15702,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15772,7 +15781,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15851,7 +15860,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -15930,7 +15939,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16009,7 +16018,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16088,7 +16097,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16169,7 +16178,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16250,7 +16259,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16329,7 +16338,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16408,7 +16417,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16487,7 +16496,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16566,7 +16575,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16645,7 +16654,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16727,7 +16736,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16806,7 +16815,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -16885,7 +16894,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -16964,7 +16973,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17043,7 +17052,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17124,7 +17133,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17205,7 +17214,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17284,7 +17293,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17363,7 +17372,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17442,7 +17451,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17521,7 +17530,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17600,7 +17609,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17679,7 +17688,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17758,7 +17767,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17837,7 +17846,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -17916,7 +17925,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -17995,7 +18004,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18076,7 +18085,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18155,7 +18164,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18234,7 +18243,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18313,7 +18322,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18392,7 +18401,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18471,7 +18480,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18550,7 +18559,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18629,7 +18638,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18708,7 +18717,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18787,7 +18796,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -18866,7 +18875,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -18945,7 +18954,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19024,7 +19033,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19103,7 +19112,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19182,7 +19191,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19261,7 +19270,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19340,7 +19349,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19419,7 +19428,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19500,7 +19509,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19579,7 +19588,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19661,7 +19670,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19743,7 +19752,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19822,7 +19831,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -19901,7 +19910,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -19982,7 +19991,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20061,7 +20070,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20140,7 +20149,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20219,7 +20228,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20298,7 +20307,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20377,7 +20386,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20458,7 +20467,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20537,7 +20546,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20616,7 +20625,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20697,7 +20706,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20778,7 +20787,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20859,7 +20868,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -20942,7 +20951,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21023,7 +21032,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21104,7 +21113,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21185,7 +21194,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21266,7 +21275,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21347,7 +21356,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21430,7 +21439,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21513,7 +21522,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21596,7 +21605,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21679,7 +21688,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21760,7 +21769,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21841,7 +21850,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -21924,7 +21933,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22003,7 +22012,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22082,7 +22091,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22161,7 +22170,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22240,7 +22249,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22319,7 +22328,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22400,7 +22409,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22479,7 +22488,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22558,7 +22567,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22637,7 +22646,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22716,7 +22725,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22795,7 +22804,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -22876,7 +22885,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -22955,7 +22964,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23034,7 +23043,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23115,7 +23124,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23194,7 +23203,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23273,7 +23282,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23352,7 +23361,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23431,7 +23440,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23510,7 +23519,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23589,7 +23598,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23668,7 +23677,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23747,7 +23756,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23828,7 +23837,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -23907,7 +23916,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -23986,7 +23995,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24065,7 +24074,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24144,7 +24153,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24223,7 +24232,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24302,7 +24311,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24381,7 +24390,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24460,7 +24469,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24539,7 +24548,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24618,7 +24627,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24697,7 +24706,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24776,7 +24785,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24858,7 +24867,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -24937,7 +24946,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25016,7 +25025,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25095,7 +25104,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25174,7 +25183,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25253,7 +25262,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25332,7 +25341,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25411,7 +25420,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25490,7 +25499,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25569,7 +25578,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25648,7 +25657,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25727,7 +25736,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25806,7 +25815,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -25885,7 +25894,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -25964,7 +25973,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26043,7 +26052,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26122,7 +26131,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26201,7 +26210,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26280,7 +26289,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26359,7 +26368,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26438,7 +26447,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26517,7 +26526,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26596,7 +26605,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26675,7 +26684,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26754,7 +26763,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26833,7 +26842,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -26912,7 +26921,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -26991,7 +27000,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27070,7 +27079,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27149,7 +27158,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27228,7 +27237,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27307,7 +27316,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27386,7 +27395,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27465,7 +27474,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27544,7 +27553,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27623,7 +27632,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27702,7 +27711,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27781,7 +27790,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -27860,7 +27869,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -27939,7 +27948,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28018,7 +28027,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28097,7 +28106,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28176,7 +28185,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28255,7 +28264,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28334,7 +28343,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28413,7 +28422,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28492,7 +28501,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28571,7 +28580,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28650,7 +28659,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28729,7 +28738,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28808,7 +28817,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -28887,7 +28896,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -28966,7 +28975,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29045,7 +29054,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29124,7 +29133,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29203,7 +29212,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29282,7 +29291,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29361,7 +29370,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:55</v>
+        <v>01:00</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Refactor API components and enhance subscription management: Update ApiRequestHandler for improved error handling and response structure, refine PremiumPlanService with better caching and API interaction, and enhance AIModelRegistry for clearer model management. Update calendar component for improved code consistency.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09F32D22-F5A6-44FD-81FA-90E5497223C3}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CCFE37C-B670-4A3E-B71B-AFEDFBD76204}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1536" uniqueCount="914">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1537" uniqueCount="915">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5334,6 +5334,10 @@
   </si>
   <si>
     <t>Found 101 errors in 26 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 89 errors in 20 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6106,7 +6110,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D18"/>
+  <dimension ref="B2:D19"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6204,6 +6208,11 @@
     <row r="18" spans="3:3">
       <c r="C18" t="s">
         <v>913</v>
+      </c>
+    </row>
+    <row r="19" spans="3:3">
+      <c r="C19" t="s">
+        <v>914</v>
       </c>
     </row>
   </sheetData>
@@ -6370,7 +6379,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6381,7 +6390,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>01:04</v>
+        <v>01:08</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6580,7 +6589,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6659,7 +6668,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6738,7 +6747,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6817,7 +6826,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -6896,7 +6905,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -6975,7 +6984,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7054,7 +7063,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7133,7 +7142,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7212,7 +7221,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7291,7 +7300,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7370,7 +7379,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7449,7 +7458,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7528,7 +7537,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7607,7 +7616,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7686,7 +7695,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7765,7 +7774,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7844,7 +7853,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -7923,7 +7932,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8002,7 +8011,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8081,7 +8090,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8160,7 +8169,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8239,7 +8248,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8318,7 +8327,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8397,7 +8406,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8476,7 +8485,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8557,7 +8566,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8638,7 +8647,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8719,7 +8728,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8798,7 +8807,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -8877,7 +8886,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -8956,7 +8965,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9037,7 +9046,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9118,7 +9127,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9199,7 +9208,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9278,7 +9287,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9357,7 +9366,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9436,7 +9445,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9515,7 +9524,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9594,7 +9603,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9675,7 +9684,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9756,7 +9765,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9835,7 +9844,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -9914,7 +9923,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -9993,7 +10002,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10072,7 +10081,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10151,7 +10160,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10232,7 +10241,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10313,7 +10322,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10392,7 +10401,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10471,7 +10480,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10550,7 +10559,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10629,7 +10638,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10708,7 +10717,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10789,7 +10798,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10868,7 +10877,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -10949,7 +10958,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11028,7 +11037,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11107,7 +11116,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11186,7 +11195,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11265,7 +11274,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11344,7 +11353,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11425,7 +11434,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11504,7 +11513,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11583,7 +11592,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11665,7 +11674,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11744,7 +11753,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11823,7 +11832,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -11902,7 +11911,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -11981,7 +11990,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12060,7 +12069,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12139,7 +12148,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12218,7 +12227,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12297,7 +12306,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12376,7 +12385,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12455,7 +12464,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12534,7 +12543,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12613,7 +12622,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12692,7 +12701,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12771,7 +12780,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12850,7 +12859,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -12929,7 +12938,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13008,7 +13017,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13087,7 +13096,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13166,7 +13175,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13245,7 +13254,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13324,7 +13333,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13403,7 +13412,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13482,7 +13491,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13561,7 +13570,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13640,7 +13649,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13719,7 +13728,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13798,7 +13807,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -13877,7 +13886,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -13956,7 +13965,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14035,7 +14044,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14114,7 +14123,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14193,7 +14202,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14274,7 +14283,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14353,7 +14362,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14432,7 +14441,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14511,7 +14520,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14590,7 +14599,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14669,7 +14678,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14750,7 +14759,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14831,7 +14840,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -14910,7 +14919,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -14989,7 +14998,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15068,7 +15077,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15147,7 +15156,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15228,7 +15237,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15307,7 +15316,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15386,7 +15395,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15465,7 +15474,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15544,7 +15553,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15623,7 +15632,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15702,7 +15711,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15781,7 +15790,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15860,7 +15869,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -15939,7 +15948,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16018,7 +16027,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16097,7 +16106,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16178,7 +16187,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16259,7 +16268,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16338,7 +16347,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16417,7 +16426,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16496,7 +16505,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16575,7 +16584,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16654,7 +16663,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16736,7 +16745,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16815,7 +16824,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -16894,7 +16903,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -16973,7 +16982,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17052,7 +17061,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17133,7 +17142,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17214,7 +17223,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17293,7 +17302,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17372,7 +17381,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17451,7 +17460,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17530,7 +17539,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17609,7 +17618,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17688,7 +17697,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17767,7 +17776,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17846,7 +17855,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -17925,7 +17934,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18004,7 +18013,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18085,7 +18094,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18164,7 +18173,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18243,7 +18252,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18322,7 +18331,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18401,7 +18410,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18480,7 +18489,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18559,7 +18568,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18638,7 +18647,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18717,7 +18726,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18796,7 +18805,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -18875,7 +18884,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -18954,7 +18963,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19033,7 +19042,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19112,7 +19121,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19191,7 +19200,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19270,7 +19279,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19349,7 +19358,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19428,7 +19437,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19509,7 +19518,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19588,7 +19597,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19670,7 +19679,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19752,7 +19761,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19831,7 +19840,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -19910,7 +19919,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -19991,7 +20000,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20070,7 +20079,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20149,7 +20158,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20228,7 +20237,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20307,7 +20316,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20386,7 +20395,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20467,7 +20476,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20546,7 +20555,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20625,7 +20634,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20706,7 +20715,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20787,7 +20796,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20868,7 +20877,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -20951,7 +20960,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21032,7 +21041,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21113,7 +21122,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21194,7 +21203,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21275,7 +21284,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21356,7 +21365,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21439,7 +21448,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21522,7 +21531,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21605,7 +21614,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21688,7 +21697,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21769,7 +21778,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21850,7 +21859,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -21933,7 +21942,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22012,7 +22021,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22091,7 +22100,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22170,7 +22179,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22249,7 +22258,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22328,7 +22337,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22409,7 +22418,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22488,7 +22497,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22567,7 +22576,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22646,7 +22655,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22725,7 +22734,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22804,7 +22813,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -22885,7 +22894,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -22964,7 +22973,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23043,7 +23052,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23124,7 +23133,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23203,7 +23212,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23282,7 +23291,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23361,7 +23370,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23440,7 +23449,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23519,7 +23528,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23598,7 +23607,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23677,7 +23686,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23756,7 +23765,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23837,7 +23846,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -23916,7 +23925,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -23995,7 +24004,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24074,7 +24083,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24153,7 +24162,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24232,7 +24241,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24311,7 +24320,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24390,7 +24399,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24469,7 +24478,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24548,7 +24557,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24627,7 +24636,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24706,7 +24715,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24785,7 +24794,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24867,7 +24876,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -24946,7 +24955,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25025,7 +25034,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25104,7 +25113,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25183,7 +25192,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25262,7 +25271,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25341,7 +25350,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25420,7 +25429,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25499,7 +25508,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25578,7 +25587,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25657,7 +25666,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25736,7 +25745,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25815,7 +25824,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -25894,7 +25903,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -25973,7 +25982,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26052,7 +26061,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26131,7 +26140,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26210,7 +26219,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26289,7 +26298,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26368,7 +26377,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26447,7 +26456,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26526,7 +26535,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26605,7 +26614,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26684,7 +26693,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26763,7 +26772,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26842,7 +26851,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -26921,7 +26930,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27000,7 +27009,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27079,7 +27088,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27158,7 +27167,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27237,7 +27246,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27316,7 +27325,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27395,7 +27404,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27474,7 +27483,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27553,7 +27562,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27632,7 +27641,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27711,7 +27720,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27790,7 +27799,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -27869,7 +27878,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -27948,7 +27957,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28027,7 +28036,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28106,7 +28115,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28185,7 +28194,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28264,7 +28273,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28343,7 +28352,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28422,7 +28431,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28501,7 +28510,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28580,7 +28589,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28659,7 +28668,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28738,7 +28747,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28817,7 +28826,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -28896,7 +28905,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -28975,7 +28984,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29054,7 +29063,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29133,7 +29142,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29212,7 +29221,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29291,7 +29300,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29370,7 +29379,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:00</v>
+        <v>01:05</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Refactor API client components: Update ApiClientHttpMethods to separate request configuration properties, enhance ApiPlugin with new PluginHooks interface, and modify import paths for better clarity. Update ExtendedRequestConfig to use RequestPriority type.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CCFE37C-B670-4A3E-B71B-AFEDFBD76204}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7EE54340-E54A-421B-B29B-BE15F35AB19F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1537" uniqueCount="915">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1538" uniqueCount="916">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5338,6 +5338,10 @@
   </si>
   <si>
     <t>Found 89 errors in 20 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 74 errors in 18 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6110,7 +6114,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D19"/>
+  <dimension ref="B2:D20"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6213,6 +6217,11 @@
     <row r="19" spans="3:3">
       <c r="C19" t="s">
         <v>914</v>
+      </c>
+    </row>
+    <row r="20" spans="3:3">
+      <c r="C20" t="s">
+        <v>915</v>
       </c>
     </row>
   </sheetData>
@@ -6379,7 +6388,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6390,7 +6399,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>01:08</v>
+        <v>01:12</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6589,7 +6598,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6668,7 +6677,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6747,7 +6756,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6826,7 +6835,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -6905,7 +6914,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -6984,7 +6993,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7063,7 +7072,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7142,7 +7151,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7221,7 +7230,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7300,7 +7309,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7379,7 +7388,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7458,7 +7467,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7537,7 +7546,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7616,7 +7625,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7695,7 +7704,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7774,7 +7783,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7853,7 +7862,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -7932,7 +7941,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8011,7 +8020,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8090,7 +8099,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8169,7 +8178,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8248,7 +8257,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8327,7 +8336,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8406,7 +8415,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8485,7 +8494,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8566,7 +8575,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8647,7 +8656,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8728,7 +8737,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8807,7 +8816,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -8886,7 +8895,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -8965,7 +8974,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9046,7 +9055,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9127,7 +9136,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9208,7 +9217,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9287,7 +9296,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9366,7 +9375,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9445,7 +9454,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9524,7 +9533,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9603,7 +9612,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9684,7 +9693,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9765,7 +9774,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9844,7 +9853,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -9923,7 +9932,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10002,7 +10011,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10081,7 +10090,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10160,7 +10169,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10241,7 +10250,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10322,7 +10331,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10401,7 +10410,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10480,7 +10489,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10559,7 +10568,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10638,7 +10647,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10717,7 +10726,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10798,7 +10807,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10877,7 +10886,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -10958,7 +10967,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11037,7 +11046,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11116,7 +11125,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11195,7 +11204,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11274,7 +11283,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11353,7 +11362,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11434,7 +11443,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11513,7 +11522,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11592,7 +11601,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11674,7 +11683,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11753,7 +11762,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11832,7 +11841,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -11911,7 +11920,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -11990,7 +11999,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12069,7 +12078,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12148,7 +12157,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12227,7 +12236,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12306,7 +12315,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12385,7 +12394,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12464,7 +12473,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12543,7 +12552,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12622,7 +12631,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12701,7 +12710,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12780,7 +12789,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12859,7 +12868,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -12938,7 +12947,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13017,7 +13026,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13096,7 +13105,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13175,7 +13184,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13254,7 +13263,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13333,7 +13342,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13412,7 +13421,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13491,7 +13500,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13570,7 +13579,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13649,7 +13658,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13728,7 +13737,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13807,7 +13816,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -13886,7 +13895,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -13965,7 +13974,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14044,7 +14053,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14123,7 +14132,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14202,7 +14211,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14283,7 +14292,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14362,7 +14371,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14441,7 +14450,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14520,7 +14529,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14599,7 +14608,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14678,7 +14687,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14759,7 +14768,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14840,7 +14849,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -14919,7 +14928,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -14998,7 +15007,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15077,7 +15086,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15156,7 +15165,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15237,7 +15246,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15316,7 +15325,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15395,7 +15404,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15474,7 +15483,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15553,7 +15562,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15632,7 +15641,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15711,7 +15720,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15790,7 +15799,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15869,7 +15878,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -15948,7 +15957,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16027,7 +16036,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16106,7 +16115,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16187,7 +16196,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16268,7 +16277,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16347,7 +16356,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16426,7 +16435,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16505,7 +16514,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16584,7 +16593,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16663,7 +16672,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16745,7 +16754,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16824,7 +16833,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -16903,7 +16912,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -16982,7 +16991,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17061,7 +17070,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17142,7 +17151,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17223,7 +17232,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17302,7 +17311,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17381,7 +17390,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17460,7 +17469,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17539,7 +17548,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17618,7 +17627,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17697,7 +17706,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17776,7 +17785,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17855,7 +17864,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -17934,7 +17943,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18013,7 +18022,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18094,7 +18103,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18173,7 +18182,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18252,7 +18261,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18331,7 +18340,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18410,7 +18419,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18489,7 +18498,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18568,7 +18577,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18647,7 +18656,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18726,7 +18735,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18805,7 +18814,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -18884,7 +18893,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -18963,7 +18972,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19042,7 +19051,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19121,7 +19130,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19200,7 +19209,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19279,7 +19288,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19358,7 +19367,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19437,7 +19446,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19518,7 +19527,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19597,7 +19606,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19679,7 +19688,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19761,7 +19770,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19840,7 +19849,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -19919,7 +19928,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20000,7 +20009,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20079,7 +20088,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20158,7 +20167,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20237,7 +20246,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20316,7 +20325,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20395,7 +20404,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20476,7 +20485,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20555,7 +20564,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20634,7 +20643,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20715,7 +20724,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20796,7 +20805,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20877,7 +20886,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -20960,7 +20969,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21041,7 +21050,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21122,7 +21131,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21203,7 +21212,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21284,7 +21293,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21365,7 +21374,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21448,7 +21457,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21531,7 +21540,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21614,7 +21623,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21697,7 +21706,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21778,7 +21787,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21859,7 +21868,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -21942,7 +21951,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22021,7 +22030,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22100,7 +22109,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22179,7 +22188,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22258,7 +22267,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22337,7 +22346,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22418,7 +22427,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22497,7 +22506,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22576,7 +22585,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22655,7 +22664,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22734,7 +22743,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22813,7 +22822,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -22894,7 +22903,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -22973,7 +22982,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23052,7 +23061,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23133,7 +23142,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23212,7 +23221,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23291,7 +23300,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23370,7 +23379,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23449,7 +23458,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23528,7 +23537,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23607,7 +23616,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23686,7 +23695,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23765,7 +23774,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23846,7 +23855,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -23925,7 +23934,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24004,7 +24013,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24083,7 +24092,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24162,7 +24171,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24241,7 +24250,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24320,7 +24329,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24399,7 +24408,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24478,7 +24487,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24557,7 +24566,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24636,7 +24645,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24715,7 +24724,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24794,7 +24803,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24876,7 +24885,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -24955,7 +24964,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25034,7 +25043,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25113,7 +25122,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25192,7 +25201,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25271,7 +25280,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25350,7 +25359,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25429,7 +25438,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25508,7 +25517,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25587,7 +25596,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25666,7 +25675,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25745,7 +25754,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25824,7 +25833,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -25903,7 +25912,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -25982,7 +25991,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26061,7 +26070,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26140,7 +26149,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26219,7 +26228,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26298,7 +26307,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26377,7 +26386,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26456,7 +26465,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26535,7 +26544,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26614,7 +26623,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26693,7 +26702,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26772,7 +26781,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26851,7 +26860,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -26930,7 +26939,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27009,7 +27018,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27088,7 +27097,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27167,7 +27176,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27246,7 +27255,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27325,7 +27334,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27404,7 +27413,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27483,7 +27492,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27562,7 +27571,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27641,7 +27650,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27720,7 +27729,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27799,7 +27808,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -27878,7 +27887,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -27957,7 +27966,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28036,7 +28045,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28115,7 +28124,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28194,7 +28203,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28273,7 +28282,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28352,7 +28361,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28431,7 +28440,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28510,7 +28519,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28589,7 +28598,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28668,7 +28677,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28747,7 +28756,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28826,7 +28835,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -28905,7 +28914,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -28984,7 +28993,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29063,7 +29072,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29142,7 +29151,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29221,7 +29230,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29300,7 +29309,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29379,7 +29388,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:05</v>
+        <v>01:10</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Enhance ApiRequestExecutor: Introduce priority mapping for queued requests, improve processing time handling in response metadata, and update related code for better clarity and maintainability. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7EE54340-E54A-421B-B29B-BE15F35AB19F}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DCDB1AAB-A003-4583-BAA9-1606A15D15FB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1538" uniqueCount="916">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1539" uniqueCount="917">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5342,6 +5342,10 @@
   </si>
   <si>
     <t>Found 74 errors in 18 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 68 errors in 18 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6114,7 +6118,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D20"/>
+  <dimension ref="B2:D21"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6222,6 +6226,11 @@
     <row r="20" spans="3:3">
       <c r="C20" t="s">
         <v>915</v>
+      </c>
+    </row>
+    <row r="21" spans="3:3">
+      <c r="C21" t="s">
+        <v>916</v>
       </c>
     </row>
   </sheetData>
@@ -6388,7 +6397,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6399,7 +6408,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>01:12</v>
+        <v>01:16</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6598,7 +6607,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6677,7 +6686,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6756,7 +6765,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6835,7 +6844,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -6914,7 +6923,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -6993,7 +7002,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7072,7 +7081,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7151,7 +7160,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7230,7 +7239,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7309,7 +7318,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7388,7 +7397,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7467,7 +7476,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7546,7 +7555,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7625,7 +7634,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7704,7 +7713,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7783,7 +7792,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7862,7 +7871,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -7941,7 +7950,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8020,7 +8029,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8099,7 +8108,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8178,7 +8187,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8257,7 +8266,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8336,7 +8345,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8415,7 +8424,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8494,7 +8503,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8575,7 +8584,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8656,7 +8665,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8737,7 +8746,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8816,7 +8825,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -8895,7 +8904,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -8974,7 +8983,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9055,7 +9064,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9136,7 +9145,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9217,7 +9226,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9296,7 +9305,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9375,7 +9384,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9454,7 +9463,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9533,7 +9542,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9612,7 +9621,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9693,7 +9702,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9774,7 +9783,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9853,7 +9862,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -9932,7 +9941,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10011,7 +10020,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10090,7 +10099,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10169,7 +10178,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10250,7 +10259,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10331,7 +10340,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10410,7 +10419,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10489,7 +10498,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10568,7 +10577,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10647,7 +10656,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10726,7 +10735,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10807,7 +10816,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10886,7 +10895,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -10967,7 +10976,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11046,7 +11055,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11125,7 +11134,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11204,7 +11213,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11283,7 +11292,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11362,7 +11371,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11443,7 +11452,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11522,7 +11531,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11601,7 +11610,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11683,7 +11692,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11762,7 +11771,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11841,7 +11850,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -11920,7 +11929,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -11999,7 +12008,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12078,7 +12087,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12157,7 +12166,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12236,7 +12245,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12315,7 +12324,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12394,7 +12403,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12473,7 +12482,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12552,7 +12561,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12631,7 +12640,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12710,7 +12719,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12789,7 +12798,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12868,7 +12877,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -12947,7 +12956,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13026,7 +13035,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13105,7 +13114,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13184,7 +13193,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13263,7 +13272,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13342,7 +13351,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13421,7 +13430,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13500,7 +13509,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13579,7 +13588,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13658,7 +13667,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13737,7 +13746,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13816,7 +13825,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -13895,7 +13904,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -13974,7 +13983,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14053,7 +14062,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14132,7 +14141,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14211,7 +14220,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14292,7 +14301,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14371,7 +14380,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14450,7 +14459,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14529,7 +14538,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14608,7 +14617,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14687,7 +14696,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14768,7 +14777,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14849,7 +14858,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -14928,7 +14937,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -15007,7 +15016,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15086,7 +15095,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15165,7 +15174,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15246,7 +15255,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15325,7 +15334,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15404,7 +15413,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15483,7 +15492,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15562,7 +15571,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15641,7 +15650,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15720,7 +15729,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15799,7 +15808,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15878,7 +15887,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -15957,7 +15966,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16036,7 +16045,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16115,7 +16124,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16196,7 +16205,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16277,7 +16286,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16356,7 +16365,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16435,7 +16444,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16514,7 +16523,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16593,7 +16602,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16672,7 +16681,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16754,7 +16763,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16833,7 +16842,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -16912,7 +16921,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -16991,7 +17000,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17070,7 +17079,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17151,7 +17160,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17232,7 +17241,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17311,7 +17320,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17390,7 +17399,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17469,7 +17478,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17548,7 +17557,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17627,7 +17636,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17706,7 +17715,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17785,7 +17794,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17864,7 +17873,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -17943,7 +17952,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18022,7 +18031,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18103,7 +18112,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18182,7 +18191,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18261,7 +18270,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18340,7 +18349,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18419,7 +18428,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18498,7 +18507,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18577,7 +18586,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18656,7 +18665,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18735,7 +18744,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18814,7 +18823,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -18893,7 +18902,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -18972,7 +18981,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19051,7 +19060,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19130,7 +19139,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19209,7 +19218,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19288,7 +19297,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19367,7 +19376,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19446,7 +19455,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19527,7 +19536,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19606,7 +19615,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19688,7 +19697,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19770,7 +19779,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19849,7 +19858,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -19928,7 +19937,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20009,7 +20018,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20088,7 +20097,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20167,7 +20176,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20246,7 +20255,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20325,7 +20334,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20404,7 +20413,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20485,7 +20494,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20564,7 +20573,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20643,7 +20652,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20724,7 +20733,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20805,7 +20814,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20886,7 +20895,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -20969,7 +20978,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21050,7 +21059,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21131,7 +21140,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21212,7 +21221,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21293,7 +21302,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21374,7 +21383,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21457,7 +21466,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21540,7 +21549,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21623,7 +21632,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21706,7 +21715,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21787,7 +21796,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21868,7 +21877,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -21951,7 +21960,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22030,7 +22039,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22109,7 +22118,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22188,7 +22197,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22267,7 +22276,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22346,7 +22355,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22427,7 +22436,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22506,7 +22515,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22585,7 +22594,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22664,7 +22673,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22743,7 +22752,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22822,7 +22831,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -22903,7 +22912,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -22982,7 +22991,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23061,7 +23070,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23142,7 +23151,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23221,7 +23230,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23300,7 +23309,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23379,7 +23388,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23458,7 +23467,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23537,7 +23546,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23616,7 +23625,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23695,7 +23704,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23774,7 +23783,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23855,7 +23864,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -23934,7 +23943,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24013,7 +24022,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24092,7 +24101,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24171,7 +24180,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24250,7 +24259,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24329,7 +24338,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24408,7 +24417,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24487,7 +24496,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24566,7 +24575,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24645,7 +24654,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24724,7 +24733,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24803,7 +24812,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24885,7 +24894,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -24964,7 +24973,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25043,7 +25052,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25122,7 +25131,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25201,7 +25210,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25280,7 +25289,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25359,7 +25368,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25438,7 +25447,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25517,7 +25526,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25596,7 +25605,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25675,7 +25684,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25754,7 +25763,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25833,7 +25842,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -25912,7 +25921,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -25991,7 +26000,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26070,7 +26079,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26149,7 +26158,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26228,7 +26237,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26307,7 +26316,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26386,7 +26395,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26465,7 +26474,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26544,7 +26553,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26623,7 +26632,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26702,7 +26711,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26781,7 +26790,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26860,7 +26869,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -26939,7 +26948,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27018,7 +27027,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27097,7 +27106,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27176,7 +27185,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27255,7 +27264,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27334,7 +27343,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27413,7 +27422,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27492,7 +27501,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27571,7 +27580,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27650,7 +27659,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27729,7 +27738,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27808,7 +27817,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -27887,7 +27896,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -27966,7 +27975,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28045,7 +28054,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28124,7 +28133,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28203,7 +28212,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28282,7 +28291,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28361,7 +28370,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28440,7 +28449,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28519,7 +28528,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28598,7 +28607,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28677,7 +28686,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28756,7 +28765,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28835,7 +28844,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -28914,7 +28923,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -28993,7 +29002,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29072,7 +29081,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29151,7 +29160,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29230,7 +29239,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29309,7 +29318,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29388,7 +29397,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:10</v>
+        <v>01:15</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Refactor ApiRequestHandler: Improve handling of service names in plugin hooks and enhance type safety for request headers. Add UserSubscriptionInfo interface to better manage user subscription data. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DCDB1AAB-A003-4583-BAA9-1606A15D15FB}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AC47CEF-5545-4C30-AAEB-10DA74AC6478}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1539" uniqueCount="917">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1540" uniqueCount="918">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5346,6 +5346,10 @@
   </si>
   <si>
     <t>Found 68 errors in 18 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 67 errors in 17 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6118,7 +6122,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D21"/>
+  <dimension ref="B2:D22"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6231,6 +6235,11 @@
     <row r="21" spans="3:3">
       <c r="C21" t="s">
         <v>916</v>
+      </c>
+    </row>
+    <row r="22" spans="3:3">
+      <c r="C22" t="s">
+        <v>917</v>
       </c>
     </row>
   </sheetData>
@@ -6397,7 +6406,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6408,7 +6417,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>01:16</v>
+        <v>01:21</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6607,7 +6616,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6686,7 +6695,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6765,7 +6774,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6844,7 +6853,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -6923,7 +6932,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -7002,7 +7011,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7081,7 +7090,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7160,7 +7169,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7239,7 +7248,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7318,7 +7327,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7397,7 +7406,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7476,7 +7485,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7555,7 +7564,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7634,7 +7643,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7713,7 +7722,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7792,7 +7801,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7871,7 +7880,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -7950,7 +7959,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8029,7 +8038,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8108,7 +8117,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8187,7 +8196,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8266,7 +8275,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8345,7 +8354,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8424,7 +8433,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8503,7 +8512,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8584,7 +8593,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8665,7 +8674,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8746,7 +8755,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8825,7 +8834,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -8904,7 +8913,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -8983,7 +8992,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9064,7 +9073,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9145,7 +9154,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9226,7 +9235,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9305,7 +9314,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9384,7 +9393,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9463,7 +9472,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9542,7 +9551,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9621,7 +9630,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9702,7 +9711,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9783,7 +9792,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9862,7 +9871,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -9941,7 +9950,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10020,7 +10029,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10099,7 +10108,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10178,7 +10187,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10259,7 +10268,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10340,7 +10349,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10419,7 +10428,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10498,7 +10507,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10577,7 +10586,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10656,7 +10665,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10735,7 +10744,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10816,7 +10825,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10895,7 +10904,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -10976,7 +10985,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11055,7 +11064,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11134,7 +11143,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11213,7 +11222,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11292,7 +11301,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11371,7 +11380,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11452,7 +11461,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11531,7 +11540,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11610,7 +11619,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11692,7 +11701,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11771,7 +11780,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11850,7 +11859,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -11929,7 +11938,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -12008,7 +12017,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12087,7 +12096,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12166,7 +12175,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12245,7 +12254,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12324,7 +12333,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12403,7 +12412,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12482,7 +12491,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12561,7 +12570,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12640,7 +12649,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12719,7 +12728,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12798,7 +12807,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12877,7 +12886,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -12956,7 +12965,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13035,7 +13044,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13114,7 +13123,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13193,7 +13202,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13272,7 +13281,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13351,7 +13360,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13430,7 +13439,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13509,7 +13518,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13588,7 +13597,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13667,7 +13676,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13746,7 +13755,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13825,7 +13834,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -13904,7 +13913,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -13983,7 +13992,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14062,7 +14071,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14141,7 +14150,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14220,7 +14229,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14301,7 +14310,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14380,7 +14389,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14459,7 +14468,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14538,7 +14547,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14617,7 +14626,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14696,7 +14705,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14777,7 +14786,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14858,7 +14867,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -14937,7 +14946,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -15016,7 +15025,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15095,7 +15104,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15174,7 +15183,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15255,7 +15264,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15334,7 +15343,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15413,7 +15422,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15492,7 +15501,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15571,7 +15580,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15650,7 +15659,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15729,7 +15738,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15808,7 +15817,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15887,7 +15896,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -15966,7 +15975,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16045,7 +16054,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16124,7 +16133,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16205,7 +16214,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16286,7 +16295,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16365,7 +16374,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16444,7 +16453,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16523,7 +16532,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16602,7 +16611,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16681,7 +16690,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16763,7 +16772,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16842,7 +16851,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -16921,7 +16930,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -17000,7 +17009,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17079,7 +17088,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17160,7 +17169,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17241,7 +17250,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17320,7 +17329,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17399,7 +17408,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17478,7 +17487,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17557,7 +17566,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17636,7 +17645,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17715,7 +17724,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17794,7 +17803,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17873,7 +17882,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -17952,7 +17961,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18031,7 +18040,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18112,7 +18121,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18191,7 +18200,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18270,7 +18279,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18349,7 +18358,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18428,7 +18437,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18507,7 +18516,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18586,7 +18595,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18665,7 +18674,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18744,7 +18753,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18823,7 +18832,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -18902,7 +18911,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -18981,7 +18990,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19060,7 +19069,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19139,7 +19148,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19218,7 +19227,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19297,7 +19306,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19376,7 +19385,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19455,7 +19464,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19536,7 +19545,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19615,7 +19624,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19697,7 +19706,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19779,7 +19788,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19858,7 +19867,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -19937,7 +19946,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20018,7 +20027,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20097,7 +20106,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20176,7 +20185,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20255,7 +20264,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20334,7 +20343,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20413,7 +20422,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20494,7 +20503,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20573,7 +20582,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20652,7 +20661,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20733,7 +20742,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20814,7 +20823,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20895,7 +20904,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -20978,7 +20987,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21059,7 +21068,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21140,7 +21149,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21221,7 +21230,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21302,7 +21311,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21383,7 +21392,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21466,7 +21475,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21549,7 +21558,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21632,7 +21641,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21715,7 +21724,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21796,7 +21805,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21877,7 +21886,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -21960,7 +21969,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22039,7 +22048,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22118,7 +22127,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22197,7 +22206,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22276,7 +22285,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22355,7 +22364,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22436,7 +22445,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22515,7 +22524,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22594,7 +22603,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22673,7 +22682,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22752,7 +22761,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22831,7 +22840,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -22912,7 +22921,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -22991,7 +23000,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23070,7 +23079,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23151,7 +23160,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23230,7 +23239,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23309,7 +23318,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23388,7 +23397,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23467,7 +23476,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23546,7 +23555,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23625,7 +23634,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23704,7 +23713,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23783,7 +23792,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23864,7 +23873,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -23943,7 +23952,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24022,7 +24031,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24101,7 +24110,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24180,7 +24189,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24259,7 +24268,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24338,7 +24347,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24417,7 +24426,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24496,7 +24505,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24575,7 +24584,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24654,7 +24663,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24733,7 +24742,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24812,7 +24821,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24894,7 +24903,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -24973,7 +24982,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25052,7 +25061,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25131,7 +25140,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25210,7 +25219,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25289,7 +25298,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25368,7 +25377,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25447,7 +25456,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25526,7 +25535,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25605,7 +25614,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25684,7 +25693,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25763,7 +25772,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25842,7 +25851,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -25921,7 +25930,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -26000,7 +26009,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26079,7 +26088,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26158,7 +26167,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26237,7 +26246,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26316,7 +26325,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26395,7 +26404,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26474,7 +26483,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26553,7 +26562,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26632,7 +26641,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26711,7 +26720,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26790,7 +26799,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26869,7 +26878,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -26948,7 +26957,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27027,7 +27036,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27106,7 +27115,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27185,7 +27194,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27264,7 +27273,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27343,7 +27352,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27422,7 +27431,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27501,7 +27510,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27580,7 +27589,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27659,7 +27668,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27738,7 +27747,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27817,7 +27826,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -27896,7 +27905,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -27975,7 +27984,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28054,7 +28063,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28133,7 +28142,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28212,7 +28221,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28291,7 +28300,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28370,7 +28379,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28449,7 +28458,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28528,7 +28537,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28607,7 +28616,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28686,7 +28695,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28765,7 +28774,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28844,7 +28853,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -28923,7 +28932,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -29002,7 +29011,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29081,7 +29090,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29160,7 +29169,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29239,7 +29248,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29318,7 +29327,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29397,7 +29406,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:15</v>
+        <v>01:20</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Add SubscriptionPlan and SubscriptionData interfaces: Enhance type definitions for subscription management. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AC47CEF-5545-4C30-AAEB-10DA74AC6478}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64C4BBF7-1515-4183-BBF0-04780074AFB2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1540" uniqueCount="918">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1541" uniqueCount="919">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5350,6 +5350,10 @@
   </si>
   <si>
     <t>Found 67 errors in 17 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 64 errors in 16 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6122,7 +6126,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D22"/>
+  <dimension ref="B2:D23"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6240,6 +6244,11 @@
     <row r="22" spans="3:3">
       <c r="C22" t="s">
         <v>917</v>
+      </c>
+    </row>
+    <row r="23" spans="3:3">
+      <c r="C23" t="s">
+        <v>918</v>
       </c>
     </row>
   </sheetData>
@@ -6406,7 +6415,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6417,7 +6426,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>01:21</v>
+        <v>01:25</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6616,7 +6625,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6695,7 +6704,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6774,7 +6783,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6853,7 +6862,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -6932,7 +6941,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -7011,7 +7020,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7090,7 +7099,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7169,7 +7178,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7248,7 +7257,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7327,7 +7336,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7406,7 +7415,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7485,7 +7494,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7564,7 +7573,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7643,7 +7652,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7722,7 +7731,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7801,7 +7810,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7880,7 +7889,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -7959,7 +7968,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8038,7 +8047,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8117,7 +8126,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8196,7 +8205,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8275,7 +8284,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8354,7 +8363,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8433,7 +8442,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8512,7 +8521,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8593,7 +8602,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8674,7 +8683,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8755,7 +8764,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8834,7 +8843,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -8913,7 +8922,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -8992,7 +9001,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9073,7 +9082,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9154,7 +9163,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9235,7 +9244,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9314,7 +9323,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9393,7 +9402,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9472,7 +9481,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9551,7 +9560,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9630,7 +9639,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9711,7 +9720,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9792,7 +9801,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9871,7 +9880,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -9950,7 +9959,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10029,7 +10038,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10108,7 +10117,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10187,7 +10196,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10268,7 +10277,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10349,7 +10358,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10428,7 +10437,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10507,7 +10516,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10586,7 +10595,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10665,7 +10674,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10744,7 +10753,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10825,7 +10834,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10904,7 +10913,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -10985,7 +10994,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11064,7 +11073,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11143,7 +11152,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11222,7 +11231,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11301,7 +11310,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11380,7 +11389,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11461,7 +11470,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11540,7 +11549,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11619,7 +11628,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11701,7 +11710,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11780,7 +11789,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11859,7 +11868,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -11938,7 +11947,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -12017,7 +12026,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12096,7 +12105,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12175,7 +12184,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12254,7 +12263,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12333,7 +12342,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12412,7 +12421,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12491,7 +12500,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12570,7 +12579,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12649,7 +12658,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12728,7 +12737,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12807,7 +12816,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12886,7 +12895,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -12965,7 +12974,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13044,7 +13053,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13123,7 +13132,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13202,7 +13211,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13281,7 +13290,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13360,7 +13369,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13439,7 +13448,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13518,7 +13527,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13597,7 +13606,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13676,7 +13685,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13755,7 +13764,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13834,7 +13843,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -13913,7 +13922,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -13992,7 +14001,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14071,7 +14080,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14150,7 +14159,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14229,7 +14238,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14310,7 +14319,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14389,7 +14398,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14468,7 +14477,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14547,7 +14556,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14626,7 +14635,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14705,7 +14714,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14786,7 +14795,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14867,7 +14876,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -14946,7 +14955,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -15025,7 +15034,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15104,7 +15113,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15183,7 +15192,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15264,7 +15273,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15343,7 +15352,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15422,7 +15431,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15501,7 +15510,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15580,7 +15589,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15659,7 +15668,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15738,7 +15747,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15817,7 +15826,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15896,7 +15905,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -15975,7 +15984,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16054,7 +16063,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16133,7 +16142,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16214,7 +16223,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16295,7 +16304,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16374,7 +16383,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16453,7 +16462,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16532,7 +16541,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16611,7 +16620,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16690,7 +16699,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16772,7 +16781,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16851,7 +16860,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -16930,7 +16939,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -17009,7 +17018,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17088,7 +17097,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17169,7 +17178,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17250,7 +17259,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17329,7 +17338,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17408,7 +17417,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17487,7 +17496,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17566,7 +17575,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17645,7 +17654,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17724,7 +17733,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17803,7 +17812,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17882,7 +17891,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -17961,7 +17970,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18040,7 +18049,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18121,7 +18130,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18200,7 +18209,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18279,7 +18288,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18358,7 +18367,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18437,7 +18446,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18516,7 +18525,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18595,7 +18604,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18674,7 +18683,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18753,7 +18762,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18832,7 +18841,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -18911,7 +18920,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -18990,7 +18999,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19069,7 +19078,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19148,7 +19157,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19227,7 +19236,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19306,7 +19315,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19385,7 +19394,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19464,7 +19473,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19545,7 +19554,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19624,7 +19633,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19706,7 +19715,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19788,7 +19797,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19867,7 +19876,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -19946,7 +19955,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20027,7 +20036,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20106,7 +20115,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20185,7 +20194,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20264,7 +20273,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20343,7 +20352,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20422,7 +20431,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20503,7 +20512,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20582,7 +20591,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20661,7 +20670,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20742,7 +20751,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20823,7 +20832,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20904,7 +20913,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -20987,7 +20996,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21068,7 +21077,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21149,7 +21158,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21230,7 +21239,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21311,7 +21320,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21392,7 +21401,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21475,7 +21484,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21558,7 +21567,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21641,7 +21650,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21724,7 +21733,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21805,7 +21814,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21886,7 +21895,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -21969,7 +21978,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22048,7 +22057,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22127,7 +22136,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22206,7 +22215,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22285,7 +22294,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22364,7 +22373,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22445,7 +22454,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22524,7 +22533,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22603,7 +22612,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22682,7 +22691,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22761,7 +22770,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22840,7 +22849,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -22921,7 +22930,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -23000,7 +23009,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23079,7 +23088,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23160,7 +23169,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23239,7 +23248,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23318,7 +23327,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23397,7 +23406,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23476,7 +23485,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23555,7 +23564,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23634,7 +23643,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23713,7 +23722,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23792,7 +23801,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23873,7 +23882,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -23952,7 +23961,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24031,7 +24040,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24110,7 +24119,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24189,7 +24198,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24268,7 +24277,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24347,7 +24356,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24426,7 +24435,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24505,7 +24514,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24584,7 +24593,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24663,7 +24672,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24742,7 +24751,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24821,7 +24830,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24903,7 +24912,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -24982,7 +24991,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25061,7 +25070,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25140,7 +25149,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25219,7 +25228,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25298,7 +25307,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25377,7 +25386,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25456,7 +25465,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25535,7 +25544,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25614,7 +25623,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25693,7 +25702,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25772,7 +25781,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25851,7 +25860,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -25930,7 +25939,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -26009,7 +26018,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26088,7 +26097,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26167,7 +26176,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26246,7 +26255,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26325,7 +26334,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26404,7 +26413,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26483,7 +26492,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26562,7 +26571,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26641,7 +26650,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26720,7 +26729,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26799,7 +26808,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26878,7 +26887,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -26957,7 +26966,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27036,7 +27045,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27115,7 +27124,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27194,7 +27203,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27273,7 +27282,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27352,7 +27361,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27431,7 +27440,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27510,7 +27519,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27589,7 +27598,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27668,7 +27677,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27747,7 +27756,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27826,7 +27835,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -27905,7 +27914,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -27984,7 +27993,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28063,7 +28072,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28142,7 +28151,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28221,7 +28230,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28300,7 +28309,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28379,7 +28388,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28458,7 +28467,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28537,7 +28546,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28616,7 +28625,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28695,7 +28704,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28774,7 +28783,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28853,7 +28862,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -28932,7 +28941,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -29011,7 +29020,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29090,7 +29099,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29169,7 +29178,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29248,7 +29257,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29327,7 +29336,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29406,7 +29415,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:20</v>
+        <v>01:25</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Enhance subscription management: Add 'cancelled' status to SubscriptionStatus type, update SubscriptionInfo interface to use SubscriptionStatus, and introduce TodoHistoryItem interface for improved type safety in todo history processing. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64C4BBF7-1515-4183-BBF0-04780074AFB2}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{010239F8-1112-42A6-A678-DAF2809917FF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1541" uniqueCount="919">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1542" uniqueCount="920">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5354,6 +5354,10 @@
   </si>
   <si>
     <t>Found 64 errors in 16 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 62 errors in 15 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6126,7 +6130,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D23"/>
+  <dimension ref="B2:D24"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6249,6 +6253,11 @@
     <row r="23" spans="3:3">
       <c r="C23" t="s">
         <v>918</v>
+      </c>
+    </row>
+    <row r="24" spans="3:3">
+      <c r="C24" t="s">
+        <v>919</v>
       </c>
     </row>
   </sheetData>
@@ -6415,7 +6424,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6426,7 +6435,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6625,7 +6634,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6704,7 +6713,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6783,7 +6792,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6862,7 +6871,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -6941,7 +6950,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -7020,7 +7029,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7099,7 +7108,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7178,7 +7187,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7257,7 +7266,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7336,7 +7345,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7415,7 +7424,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7494,7 +7503,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7573,7 +7582,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7652,7 +7661,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7731,7 +7740,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7810,7 +7819,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7889,7 +7898,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -7968,7 +7977,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8047,7 +8056,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8126,7 +8135,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8205,7 +8214,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8284,7 +8293,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8363,7 +8372,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8442,7 +8451,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8521,7 +8530,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8602,7 +8611,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8683,7 +8692,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8764,7 +8773,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8843,7 +8852,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -8922,7 +8931,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -9001,7 +9010,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9082,7 +9091,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9163,7 +9172,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9244,7 +9253,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9323,7 +9332,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9402,7 +9411,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9481,7 +9490,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9560,7 +9569,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9639,7 +9648,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9720,7 +9729,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9801,7 +9810,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9880,7 +9889,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -9959,7 +9968,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10038,7 +10047,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10117,7 +10126,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10196,7 +10205,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10277,7 +10286,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10358,7 +10367,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10437,7 +10446,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10516,7 +10525,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10595,7 +10604,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10674,7 +10683,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10753,7 +10762,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10834,7 +10843,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10913,7 +10922,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -10994,7 +11003,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11073,7 +11082,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11152,7 +11161,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11231,7 +11240,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11310,7 +11319,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11389,7 +11398,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11470,7 +11479,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11549,7 +11558,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11628,7 +11637,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11710,7 +11719,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11789,7 +11798,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11868,7 +11877,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -11947,7 +11956,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -12026,7 +12035,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12105,7 +12114,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12184,7 +12193,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12263,7 +12272,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12342,7 +12351,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12421,7 +12430,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12500,7 +12509,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12579,7 +12588,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12658,7 +12667,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12737,7 +12746,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12816,7 +12825,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12895,7 +12904,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -12974,7 +12983,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13053,7 +13062,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13132,7 +13141,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13211,7 +13220,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13290,7 +13299,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13369,7 +13378,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13448,7 +13457,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13527,7 +13536,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13606,7 +13615,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13685,7 +13694,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13764,7 +13773,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13843,7 +13852,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -13922,7 +13931,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -14001,7 +14010,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14080,7 +14089,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14159,7 +14168,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14238,7 +14247,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14319,7 +14328,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14398,7 +14407,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14477,7 +14486,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14556,7 +14565,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14635,7 +14644,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14714,7 +14723,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14795,7 +14804,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14876,7 +14885,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -14955,7 +14964,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -15034,7 +15043,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15113,7 +15122,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15192,7 +15201,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15273,7 +15282,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15352,7 +15361,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15431,7 +15440,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15510,7 +15519,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15589,7 +15598,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15668,7 +15677,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15747,7 +15756,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15826,7 +15835,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15905,7 +15914,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -15984,7 +15993,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16063,7 +16072,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16142,7 +16151,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16223,7 +16232,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16304,7 +16313,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16383,7 +16392,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16462,7 +16471,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16541,7 +16550,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16620,7 +16629,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16699,7 +16708,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16781,7 +16790,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16860,7 +16869,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -16939,7 +16948,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -17018,7 +17027,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17097,7 +17106,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17178,7 +17187,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17259,7 +17268,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17338,7 +17347,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17417,7 +17426,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17496,7 +17505,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17575,7 +17584,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17654,7 +17663,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17733,7 +17742,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17812,7 +17821,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17891,7 +17900,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -17970,7 +17979,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18049,7 +18058,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18130,7 +18139,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18209,7 +18218,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18288,7 +18297,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18367,7 +18376,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18446,7 +18455,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18525,7 +18534,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18604,7 +18613,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18683,7 +18692,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18762,7 +18771,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18841,7 +18850,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -18920,7 +18929,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -18999,7 +19008,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19078,7 +19087,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19157,7 +19166,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19236,7 +19245,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19315,7 +19324,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19394,7 +19403,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19473,7 +19482,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19554,7 +19563,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19633,7 +19642,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19715,7 +19724,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19797,7 +19806,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19876,7 +19885,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -19955,7 +19964,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20036,7 +20045,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20115,7 +20124,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20194,7 +20203,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20273,7 +20282,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20352,7 +20361,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20431,7 +20440,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20512,7 +20521,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20591,7 +20600,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20670,7 +20679,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20751,7 +20760,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20832,7 +20841,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20913,7 +20922,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -20996,7 +21005,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21077,7 +21086,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21158,7 +21167,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21239,7 +21248,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21320,7 +21329,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21401,7 +21410,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21484,7 +21493,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21567,7 +21576,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21650,7 +21659,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21733,7 +21742,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21814,7 +21823,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21895,7 +21904,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -21978,7 +21987,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22057,7 +22066,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22136,7 +22145,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22215,7 +22224,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22294,7 +22303,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22373,7 +22382,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22454,7 +22463,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22533,7 +22542,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22612,7 +22621,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22691,7 +22700,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22770,7 +22779,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22849,7 +22858,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -22930,7 +22939,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -23009,7 +23018,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23088,7 +23097,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23169,7 +23178,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23248,7 +23257,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23327,7 +23336,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23406,7 +23415,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23485,7 +23494,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23564,7 +23573,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23643,7 +23652,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23722,7 +23731,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23801,7 +23810,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23882,7 +23891,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -23961,7 +23970,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24040,7 +24049,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24119,7 +24128,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24198,7 +24207,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24277,7 +24286,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24356,7 +24365,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24435,7 +24444,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24514,7 +24523,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24593,7 +24602,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24672,7 +24681,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24751,7 +24760,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24830,7 +24839,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24912,7 +24921,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -24991,7 +25000,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25070,7 +25079,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25149,7 +25158,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25228,7 +25237,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25307,7 +25316,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25386,7 +25395,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25465,7 +25474,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25544,7 +25553,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25623,7 +25632,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25702,7 +25711,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25781,7 +25790,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25860,7 +25869,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -25939,7 +25948,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -26018,7 +26027,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26097,7 +26106,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26176,7 +26185,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26255,7 +26264,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26334,7 +26343,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26413,7 +26422,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26492,7 +26501,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26571,7 +26580,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26650,7 +26659,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26729,7 +26738,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26808,7 +26817,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26887,7 +26896,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -26966,7 +26975,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27045,7 +27054,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27124,7 +27133,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27203,7 +27212,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27282,7 +27291,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27361,7 +27370,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27440,7 +27449,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27519,7 +27528,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27598,7 +27607,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27677,7 +27686,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27756,7 +27765,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27835,7 +27844,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -27914,7 +27923,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -27993,7 +28002,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28072,7 +28081,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28151,7 +28160,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28230,7 +28239,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28309,7 +28318,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28388,7 +28397,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28467,7 +28476,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28546,7 +28555,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28625,7 +28634,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28704,7 +28713,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28783,7 +28792,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28862,7 +28871,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -28941,7 +28950,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -29020,7 +29029,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29099,7 +29108,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29178,7 +29187,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29257,7 +29266,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29336,7 +29345,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29415,7 +29424,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:25</v>
+        <v>01:30</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Refactor DateRangePicker component: Enhance type safety by replacing 'any' with 'unknown' and introducing specific interfaces for date ranges and presets. Update todoRoutes to improve type handling in history processing and ensure proper initialization of DailyCounts. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{010239F8-1112-42A6-A678-DAF2809917FF}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E4A7048-251F-4F9A-A370-6ECC72A286D4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1542" uniqueCount="920">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1543" uniqueCount="921">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5358,6 +5358,10 @@
   </si>
   <si>
     <t>Found 62 errors in 15 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 63 errors in 16 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6130,7 +6134,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D24"/>
+  <dimension ref="B2:D25"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6258,6 +6262,11 @@
     <row r="24" spans="3:3">
       <c r="C24" t="s">
         <v>919</v>
+      </c>
+    </row>
+    <row r="25" spans="3:3">
+      <c r="C25" t="s">
+        <v>920</v>
       </c>
     </row>
   </sheetData>
@@ -6435,7 +6444,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>01:30</v>
+        <v>01:33</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">

</xml_diff>

<commit_message>
Refactor error handling in CachePlugin: Simplify catch blocks by removing error logging and improve type safety in usePremiumFeatures by adding expiresAt. Update DateRangePicker component to enforce required selection. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E4A7048-251F-4F9A-A370-6ECC72A286D4}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C6CDF44-8573-4EE9-90B3-D9E1DBF55244}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1543" uniqueCount="921">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1544" uniqueCount="921">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -6134,7 +6134,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D25"/>
+  <dimension ref="B2:D26"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6267,6 +6267,11 @@
     <row r="25" spans="3:3">
       <c r="C25" t="s">
         <v>920</v>
+      </c>
+    </row>
+    <row r="26" spans="3:3">
+      <c r="C26" t="s">
+        <v>918</v>
       </c>
     </row>
   </sheetData>
@@ -6433,7 +6438,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6444,7 +6449,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>01:33</v>
+        <v>01:39</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6643,7 +6648,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6722,7 +6727,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6801,7 +6806,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6880,7 +6885,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -6959,7 +6964,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -7038,7 +7043,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7117,7 +7122,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7196,7 +7201,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7275,7 +7280,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7354,7 +7359,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7433,7 +7438,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7512,7 +7517,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7591,7 +7596,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7670,7 +7675,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7749,7 +7754,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7828,7 +7833,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7907,7 +7912,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -7986,7 +7991,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8065,7 +8070,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8144,7 +8149,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8223,7 +8228,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8302,7 +8307,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8381,7 +8386,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8460,7 +8465,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8539,7 +8544,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8620,7 +8625,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8701,7 +8706,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8782,7 +8787,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8861,7 +8866,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -8940,7 +8945,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -9019,7 +9024,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9100,7 +9105,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9181,7 +9186,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9262,7 +9267,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9341,7 +9346,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9420,7 +9425,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9499,7 +9504,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9578,7 +9583,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9657,7 +9662,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9738,7 +9743,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9819,7 +9824,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9898,7 +9903,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -9977,7 +9982,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10056,7 +10061,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10135,7 +10140,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10214,7 +10219,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10295,7 +10300,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10376,7 +10381,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10455,7 +10460,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10534,7 +10539,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10613,7 +10618,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10692,7 +10697,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10771,7 +10776,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10852,7 +10857,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10931,7 +10936,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -11012,7 +11017,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11091,7 +11096,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11170,7 +11175,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11249,7 +11254,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11328,7 +11333,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11407,7 +11412,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11488,7 +11493,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11567,7 +11572,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11646,7 +11651,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11728,7 +11733,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11807,7 +11812,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11886,7 +11891,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -11965,7 +11970,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -12044,7 +12049,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12123,7 +12128,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12202,7 +12207,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12281,7 +12286,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12360,7 +12365,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12439,7 +12444,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12518,7 +12523,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12597,7 +12602,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12676,7 +12681,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12755,7 +12760,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12834,7 +12839,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12913,7 +12918,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -12992,7 +12997,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13071,7 +13076,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13150,7 +13155,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13229,7 +13234,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13308,7 +13313,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13387,7 +13392,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13466,7 +13471,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13545,7 +13550,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13624,7 +13629,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13703,7 +13708,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13782,7 +13787,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13861,7 +13866,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -13940,7 +13945,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -14019,7 +14024,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14098,7 +14103,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14177,7 +14182,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14256,7 +14261,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14337,7 +14342,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14416,7 +14421,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14495,7 +14500,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14574,7 +14579,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14653,7 +14658,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14732,7 +14737,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14813,7 +14818,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14894,7 +14899,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -14973,7 +14978,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -15052,7 +15057,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15131,7 +15136,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15210,7 +15215,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15291,7 +15296,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15370,7 +15375,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15449,7 +15454,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15528,7 +15533,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15607,7 +15612,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15686,7 +15691,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15765,7 +15770,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15844,7 +15849,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15923,7 +15928,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -16002,7 +16007,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16081,7 +16086,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16160,7 +16165,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16241,7 +16246,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16322,7 +16327,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16401,7 +16406,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16480,7 +16485,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16559,7 +16564,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16638,7 +16643,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16717,7 +16722,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16799,7 +16804,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16878,7 +16883,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -16957,7 +16962,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -17036,7 +17041,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17115,7 +17120,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17196,7 +17201,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17277,7 +17282,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17356,7 +17361,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17435,7 +17440,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17514,7 +17519,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17593,7 +17598,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17672,7 +17677,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17751,7 +17756,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17830,7 +17835,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17909,7 +17914,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -17988,7 +17993,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18067,7 +18072,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18148,7 +18153,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18227,7 +18232,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18306,7 +18311,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18385,7 +18390,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18464,7 +18469,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18543,7 +18548,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18622,7 +18627,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18701,7 +18706,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18780,7 +18785,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18859,7 +18864,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -18938,7 +18943,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -19017,7 +19022,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19096,7 +19101,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19175,7 +19180,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19254,7 +19259,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19333,7 +19338,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19412,7 +19417,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19491,7 +19496,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19572,7 +19577,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19651,7 +19656,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19733,7 +19738,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19815,7 +19820,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19894,7 +19899,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -19973,7 +19978,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20054,7 +20059,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20133,7 +20138,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20212,7 +20217,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20291,7 +20296,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20370,7 +20375,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20449,7 +20454,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20530,7 +20535,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20609,7 +20614,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20688,7 +20693,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20769,7 +20774,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20850,7 +20855,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20931,7 +20936,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -21014,7 +21019,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21095,7 +21100,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21176,7 +21181,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21257,7 +21262,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21338,7 +21343,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21419,7 +21424,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21502,7 +21507,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21585,7 +21590,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21668,7 +21673,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21751,7 +21756,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21832,7 +21837,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21913,7 +21918,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -21996,7 +22001,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22075,7 +22080,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22154,7 +22159,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22233,7 +22238,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22312,7 +22317,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22391,7 +22396,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22472,7 +22477,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22551,7 +22556,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22630,7 +22635,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22709,7 +22714,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22788,7 +22793,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22867,7 +22872,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -22948,7 +22953,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -23027,7 +23032,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23106,7 +23111,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23187,7 +23192,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23266,7 +23271,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23345,7 +23350,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23424,7 +23429,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23503,7 +23508,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23582,7 +23587,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23661,7 +23666,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23740,7 +23745,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23819,7 +23824,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23900,7 +23905,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -23979,7 +23984,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24058,7 +24063,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24137,7 +24142,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24216,7 +24221,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24295,7 +24300,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24374,7 +24379,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24453,7 +24458,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24532,7 +24537,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24611,7 +24616,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24690,7 +24695,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24769,7 +24774,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24848,7 +24853,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24930,7 +24935,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -25009,7 +25014,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25088,7 +25093,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25167,7 +25172,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25246,7 +25251,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25325,7 +25330,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25404,7 +25409,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25483,7 +25488,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25562,7 +25567,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25641,7 +25646,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25720,7 +25725,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25799,7 +25804,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25878,7 +25883,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -25957,7 +25962,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -26036,7 +26041,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26115,7 +26120,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26194,7 +26199,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26273,7 +26278,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26352,7 +26357,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26431,7 +26436,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26510,7 +26515,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26589,7 +26594,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26668,7 +26673,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26747,7 +26752,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26826,7 +26831,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26905,7 +26910,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -26984,7 +26989,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27063,7 +27068,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27142,7 +27147,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27221,7 +27226,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27300,7 +27305,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27379,7 +27384,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27458,7 +27463,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27537,7 +27542,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27616,7 +27621,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27695,7 +27700,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27774,7 +27779,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27853,7 +27858,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -27932,7 +27937,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -28011,7 +28016,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28090,7 +28095,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28169,7 +28174,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28248,7 +28253,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28327,7 +28332,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28406,7 +28411,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28485,7 +28490,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28564,7 +28569,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28643,7 +28648,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28722,7 +28727,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28801,7 +28806,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28880,7 +28885,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -28959,7 +28964,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -29038,7 +29043,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29117,7 +29122,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29196,7 +29201,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29275,7 +29280,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29354,7 +29359,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29433,7 +29438,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:30</v>
+        <v>01:35</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Refactor PremiumPlanService and NetworkMonitor: Update cache priority to MEDIUM for improved performance, enhance NetworkMonitor with online status listeners, and improve error handling in PremiumPlanService. Update CacheManager for better type safety. Update Home and PoliticalTrends components for code consistency and clarity.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C6CDF44-8573-4EE9-90B3-D9E1DBF55244}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5559AAB8-1CD9-4D76-BCA2-D303AE42D0F6}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1544" uniqueCount="921">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1545" uniqueCount="922">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5362,6 +5362,10 @@
   </si>
   <si>
     <t>Found 63 errors in 16 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 63 errors in 15 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6134,7 +6138,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D26"/>
+  <dimension ref="B2:D27"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6272,6 +6276,11 @@
     <row r="26" spans="3:3">
       <c r="C26" t="s">
         <v>918</v>
+      </c>
+    </row>
+    <row r="27" spans="3:3">
+      <c r="C27" t="s">
+        <v>921</v>
       </c>
     </row>
   </sheetData>
@@ -6438,7 +6447,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6449,7 +6458,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>01:39</v>
+        <v>01:46</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6648,7 +6657,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6727,7 +6736,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6806,7 +6815,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6885,7 +6894,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -6964,7 +6973,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -7043,7 +7052,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7122,7 +7131,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7201,7 +7210,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7280,7 +7289,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7359,7 +7368,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7438,7 +7447,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7517,7 +7526,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7596,7 +7605,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7675,7 +7684,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7754,7 +7763,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7833,7 +7842,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7912,7 +7921,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -7991,7 +8000,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8070,7 +8079,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8149,7 +8158,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8228,7 +8237,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8307,7 +8316,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8386,7 +8395,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8465,7 +8474,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8544,7 +8553,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8625,7 +8634,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8706,7 +8715,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8787,7 +8796,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8866,7 +8875,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -8945,7 +8954,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -9024,7 +9033,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9105,7 +9114,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9186,7 +9195,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9267,7 +9276,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9346,7 +9355,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9425,7 +9434,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9504,7 +9513,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9583,7 +9592,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9662,7 +9671,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9743,7 +9752,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9824,7 +9833,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9903,7 +9912,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -9982,7 +9991,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10061,7 +10070,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10140,7 +10149,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10219,7 +10228,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10300,7 +10309,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10381,7 +10390,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10460,7 +10469,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10539,7 +10548,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10618,7 +10627,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10697,7 +10706,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10776,7 +10785,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10857,7 +10866,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10936,7 +10945,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -11017,7 +11026,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11096,7 +11105,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11175,7 +11184,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11254,7 +11263,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11333,7 +11342,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11412,7 +11421,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11493,7 +11502,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11572,7 +11581,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11651,7 +11660,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11733,7 +11742,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11812,7 +11821,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11891,7 +11900,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -11970,7 +11979,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -12049,7 +12058,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12128,7 +12137,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12207,7 +12216,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12286,7 +12295,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12365,7 +12374,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12444,7 +12453,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12523,7 +12532,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12602,7 +12611,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12681,7 +12690,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12760,7 +12769,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12839,7 +12848,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12918,7 +12927,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -12997,7 +13006,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13076,7 +13085,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13155,7 +13164,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13234,7 +13243,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13313,7 +13322,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13392,7 +13401,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13471,7 +13480,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13550,7 +13559,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13629,7 +13638,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13708,7 +13717,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13787,7 +13796,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13866,7 +13875,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -13945,7 +13954,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -14024,7 +14033,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14103,7 +14112,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14182,7 +14191,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14261,7 +14270,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14342,7 +14351,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14421,7 +14430,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14500,7 +14509,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14579,7 +14588,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14658,7 +14667,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14737,7 +14746,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14818,7 +14827,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14899,7 +14908,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -14978,7 +14987,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -15057,7 +15066,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15136,7 +15145,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15215,7 +15224,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15296,7 +15305,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15375,7 +15384,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15454,7 +15463,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15533,7 +15542,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15612,7 +15621,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15691,7 +15700,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15770,7 +15779,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15849,7 +15858,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15928,7 +15937,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -16007,7 +16016,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16086,7 +16095,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16165,7 +16174,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16246,7 +16255,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16327,7 +16336,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16406,7 +16415,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16485,7 +16494,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16564,7 +16573,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16643,7 +16652,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16722,7 +16731,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16804,7 +16813,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16883,7 +16892,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -16962,7 +16971,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -17041,7 +17050,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17120,7 +17129,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17201,7 +17210,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17282,7 +17291,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17361,7 +17370,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17440,7 +17449,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17519,7 +17528,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17598,7 +17607,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17677,7 +17686,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17756,7 +17765,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17835,7 +17844,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17914,7 +17923,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -17993,7 +18002,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18072,7 +18081,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18153,7 +18162,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18232,7 +18241,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18311,7 +18320,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18390,7 +18399,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18469,7 +18478,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18548,7 +18557,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18627,7 +18636,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18706,7 +18715,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18785,7 +18794,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18864,7 +18873,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -18943,7 +18952,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -19022,7 +19031,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19101,7 +19110,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19180,7 +19189,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19259,7 +19268,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19338,7 +19347,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19417,7 +19426,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19496,7 +19505,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19577,7 +19586,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19656,7 +19665,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19738,7 +19747,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19820,7 +19829,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19899,7 +19908,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -19978,7 +19987,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20059,7 +20068,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20138,7 +20147,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20217,7 +20226,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20296,7 +20305,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20375,7 +20384,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20454,7 +20463,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20535,7 +20544,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20614,7 +20623,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20693,7 +20702,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20774,7 +20783,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20855,7 +20864,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20936,7 +20945,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -21019,7 +21028,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21100,7 +21109,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21181,7 +21190,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21262,7 +21271,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21343,7 +21352,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21424,7 +21433,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21507,7 +21516,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21590,7 +21599,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21673,7 +21682,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21756,7 +21765,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21837,7 +21846,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21918,7 +21927,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -22001,7 +22010,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22080,7 +22089,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22159,7 +22168,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22238,7 +22247,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22317,7 +22326,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22396,7 +22405,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22477,7 +22486,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22556,7 +22565,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22635,7 +22644,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22714,7 +22723,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22793,7 +22802,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22872,7 +22881,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -22953,7 +22962,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -23032,7 +23041,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23111,7 +23120,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23192,7 +23201,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23271,7 +23280,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23350,7 +23359,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23429,7 +23438,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23508,7 +23517,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23587,7 +23596,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23666,7 +23675,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23745,7 +23754,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23824,7 +23833,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23905,7 +23914,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -23984,7 +23993,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24063,7 +24072,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24142,7 +24151,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24221,7 +24230,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24300,7 +24309,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24379,7 +24388,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24458,7 +24467,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24537,7 +24546,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24616,7 +24625,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24695,7 +24704,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24774,7 +24783,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24853,7 +24862,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24935,7 +24944,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -25014,7 +25023,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25093,7 +25102,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25172,7 +25181,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25251,7 +25260,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25330,7 +25339,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25409,7 +25418,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25488,7 +25497,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25567,7 +25576,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25646,7 +25655,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25725,7 +25734,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25804,7 +25813,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25883,7 +25892,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -25962,7 +25971,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -26041,7 +26050,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26120,7 +26129,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26199,7 +26208,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26278,7 +26287,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26357,7 +26366,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26436,7 +26445,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26515,7 +26524,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26594,7 +26603,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26673,7 +26682,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26752,7 +26761,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26831,7 +26840,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26910,7 +26919,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -26989,7 +26998,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27068,7 +27077,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27147,7 +27156,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27226,7 +27235,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27305,7 +27314,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27384,7 +27393,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27463,7 +27472,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27542,7 +27551,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27621,7 +27630,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27700,7 +27709,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27779,7 +27788,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27858,7 +27867,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -27937,7 +27946,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -28016,7 +28025,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28095,7 +28104,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28174,7 +28183,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28253,7 +28262,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28332,7 +28341,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28411,7 +28420,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28490,7 +28499,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28569,7 +28578,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28648,7 +28657,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28727,7 +28736,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28806,7 +28815,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28885,7 +28894,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -28964,7 +28973,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -29043,7 +29052,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29122,7 +29131,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29201,7 +29210,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29280,7 +29289,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29359,7 +29368,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29438,7 +29447,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:35</v>
+        <v>01:45</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Refactor InviteFriendsComponent to join email addresses for invites, enhance GoogleAnalyticsProvider with better type definitions, update calendar component for improved prop handling, and modify PoliticalTrends to initialize date range as undefined. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5559AAB8-1CD9-4D76-BCA2-D303AE42D0F6}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0E3CF06-DBF0-490C-A784-0DAEBE68D2D7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1545" uniqueCount="922">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1546" uniqueCount="923">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5366,6 +5366,10 @@
   </si>
   <si>
     <t>Found 63 errors in 15 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 54 errors in 14 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6138,7 +6142,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D27"/>
+  <dimension ref="B2:D28"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6281,6 +6285,11 @@
     <row r="27" spans="3:3">
       <c r="C27" t="s">
         <v>921</v>
+      </c>
+    </row>
+    <row r="28" spans="3:3">
+      <c r="C28" t="s">
+        <v>922</v>
       </c>
     </row>
   </sheetData>
@@ -6447,7 +6456,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6458,7 +6467,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>01:46</v>
+        <v>01:52</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6657,7 +6666,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6736,7 +6745,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6815,7 +6824,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6894,7 +6903,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -6973,7 +6982,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -7052,7 +7061,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7131,7 +7140,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7210,7 +7219,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7289,7 +7298,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7368,7 +7377,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7447,7 +7456,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7526,7 +7535,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7605,7 +7614,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7684,7 +7693,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7763,7 +7772,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7842,7 +7851,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7921,7 +7930,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -8000,7 +8009,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8079,7 +8088,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8158,7 +8167,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8237,7 +8246,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8316,7 +8325,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8395,7 +8404,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8474,7 +8483,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8553,7 +8562,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8634,7 +8643,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8715,7 +8724,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8796,7 +8805,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8875,7 +8884,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -8954,7 +8963,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -9033,7 +9042,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9114,7 +9123,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9195,7 +9204,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9276,7 +9285,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9355,7 +9364,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9434,7 +9443,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9513,7 +9522,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9592,7 +9601,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9671,7 +9680,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9752,7 +9761,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9833,7 +9842,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9912,7 +9921,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -9991,7 +10000,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10070,7 +10079,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10149,7 +10158,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10228,7 +10237,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10309,7 +10318,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10390,7 +10399,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10469,7 +10478,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10548,7 +10557,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10627,7 +10636,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10706,7 +10715,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10785,7 +10794,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10866,7 +10875,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10945,7 +10954,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -11026,7 +11035,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11105,7 +11114,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11184,7 +11193,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11263,7 +11272,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11342,7 +11351,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11421,7 +11430,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11502,7 +11511,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11581,7 +11590,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11660,7 +11669,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11742,7 +11751,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11821,7 +11830,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11900,7 +11909,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -11979,7 +11988,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -12058,7 +12067,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12137,7 +12146,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12216,7 +12225,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12295,7 +12304,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12374,7 +12383,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12453,7 +12462,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12532,7 +12541,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12611,7 +12620,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12690,7 +12699,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12769,7 +12778,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12848,7 +12857,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12927,7 +12936,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -13006,7 +13015,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13085,7 +13094,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13164,7 +13173,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13243,7 +13252,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13322,7 +13331,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13401,7 +13410,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13480,7 +13489,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13559,7 +13568,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13638,7 +13647,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13717,7 +13726,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13796,7 +13805,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13875,7 +13884,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -13954,7 +13963,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -14033,7 +14042,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14112,7 +14121,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14191,7 +14200,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14270,7 +14279,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14351,7 +14360,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14430,7 +14439,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14509,7 +14518,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14588,7 +14597,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14667,7 +14676,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14746,7 +14755,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14827,7 +14836,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14908,7 +14917,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -14987,7 +14996,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -15066,7 +15075,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15145,7 +15154,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15224,7 +15233,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15305,7 +15314,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15384,7 +15393,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15463,7 +15472,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15542,7 +15551,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15621,7 +15630,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15700,7 +15709,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15779,7 +15788,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15858,7 +15867,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15937,7 +15946,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -16016,7 +16025,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16095,7 +16104,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16174,7 +16183,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16255,7 +16264,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16336,7 +16345,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16415,7 +16424,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16494,7 +16503,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16573,7 +16582,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16652,7 +16661,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16731,7 +16740,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16813,7 +16822,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16892,7 +16901,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -16971,7 +16980,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -17050,7 +17059,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17129,7 +17138,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17210,7 +17219,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17291,7 +17300,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17370,7 +17379,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17449,7 +17458,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17528,7 +17537,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17607,7 +17616,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17686,7 +17695,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17765,7 +17774,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17844,7 +17853,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17923,7 +17932,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -18002,7 +18011,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18081,7 +18090,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18162,7 +18171,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18241,7 +18250,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18320,7 +18329,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18399,7 +18408,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18478,7 +18487,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18557,7 +18566,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18636,7 +18645,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18715,7 +18724,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18794,7 +18803,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18873,7 +18882,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -18952,7 +18961,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -19031,7 +19040,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19110,7 +19119,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19189,7 +19198,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19268,7 +19277,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19347,7 +19356,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19426,7 +19435,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19505,7 +19514,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19586,7 +19595,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19665,7 +19674,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19747,7 +19756,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19829,7 +19838,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19908,7 +19917,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -19987,7 +19996,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20068,7 +20077,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20147,7 +20156,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20226,7 +20235,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20305,7 +20314,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20384,7 +20393,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20463,7 +20472,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20544,7 +20553,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20623,7 +20632,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20702,7 +20711,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20783,7 +20792,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20864,7 +20873,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20945,7 +20954,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -21028,7 +21037,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21109,7 +21118,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21190,7 +21199,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21271,7 +21280,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21352,7 +21361,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21433,7 +21442,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21516,7 +21525,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21599,7 +21608,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21682,7 +21691,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21765,7 +21774,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21846,7 +21855,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21927,7 +21936,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -22010,7 +22019,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22089,7 +22098,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22168,7 +22177,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22247,7 +22256,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22326,7 +22335,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22405,7 +22414,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22486,7 +22495,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22565,7 +22574,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22644,7 +22653,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22723,7 +22732,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22802,7 +22811,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22881,7 +22890,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -22962,7 +22971,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -23041,7 +23050,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23120,7 +23129,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23201,7 +23210,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23280,7 +23289,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23359,7 +23368,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23438,7 +23447,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23517,7 +23526,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23596,7 +23605,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23675,7 +23684,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23754,7 +23763,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23833,7 +23842,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23914,7 +23923,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -23993,7 +24002,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24072,7 +24081,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24151,7 +24160,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24230,7 +24239,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24309,7 +24318,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24388,7 +24397,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24467,7 +24476,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24546,7 +24555,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24625,7 +24634,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24704,7 +24713,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24783,7 +24792,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24862,7 +24871,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24944,7 +24953,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -25023,7 +25032,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25102,7 +25111,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25181,7 +25190,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25260,7 +25269,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25339,7 +25348,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25418,7 +25427,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25497,7 +25506,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25576,7 +25585,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25655,7 +25664,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25734,7 +25743,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25813,7 +25822,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25892,7 +25901,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -25971,7 +25980,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -26050,7 +26059,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26129,7 +26138,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26208,7 +26217,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26287,7 +26296,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26366,7 +26375,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26445,7 +26454,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26524,7 +26533,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26603,7 +26612,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26682,7 +26691,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26761,7 +26770,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26840,7 +26849,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26919,7 +26928,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -26998,7 +27007,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27077,7 +27086,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27156,7 +27165,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27235,7 +27244,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27314,7 +27323,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27393,7 +27402,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27472,7 +27481,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27551,7 +27560,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27630,7 +27639,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27709,7 +27718,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27788,7 +27797,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27867,7 +27876,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -27946,7 +27955,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -28025,7 +28034,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28104,7 +28113,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28183,7 +28192,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28262,7 +28271,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28341,7 +28350,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28420,7 +28429,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28499,7 +28508,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28578,7 +28587,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28657,7 +28666,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28736,7 +28745,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28815,7 +28824,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28894,7 +28903,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -28973,7 +28982,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -29052,7 +29061,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29131,7 +29140,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29210,7 +29219,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29289,7 +29298,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29368,7 +29377,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29447,7 +29456,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:45</v>
+        <v>01:50</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Refactor InviteFriendsComponent to improve invite handling by assuming success on user invitations, enhance type safety with InvitedUser interface, and update analytics functions for better type definitions. Modify PoliticalTrends component to streamline date range imports. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0E3CF06-DBF0-490C-A784-0DAEBE68D2D7}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0A94D47-EB38-414E-9E37-725EAC88550C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1546" uniqueCount="923">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1547" uniqueCount="924">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5370,6 +5370,10 @@
   </si>
   <si>
     <t>Found 54 errors in 14 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 56 errors in 14 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6142,7 +6146,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D28"/>
+  <dimension ref="B2:D29"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6290,6 +6294,11 @@
     <row r="28" spans="3:3">
       <c r="C28" t="s">
         <v>922</v>
+      </c>
+    </row>
+    <row r="29" spans="3:3">
+      <c r="C29" t="s">
+        <v>923</v>
       </c>
     </row>
   </sheetData>
@@ -6456,7 +6465,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6467,7 +6476,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>01:52</v>
+        <v>01:57</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6666,7 +6675,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6745,7 +6754,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6824,7 +6833,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6903,7 +6912,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -6982,7 +6991,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -7061,7 +7070,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7140,7 +7149,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7219,7 +7228,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7298,7 +7307,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7377,7 +7386,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7456,7 +7465,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7535,7 +7544,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7614,7 +7623,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7693,7 +7702,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7772,7 +7781,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7851,7 +7860,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7930,7 +7939,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -8009,7 +8018,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8088,7 +8097,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8167,7 +8176,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8246,7 +8255,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8325,7 +8334,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8404,7 +8413,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8483,7 +8492,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8562,7 +8571,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8643,7 +8652,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8724,7 +8733,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8805,7 +8814,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8884,7 +8893,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -8963,7 +8972,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -9042,7 +9051,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9123,7 +9132,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9204,7 +9213,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9285,7 +9294,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9364,7 +9373,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9443,7 +9452,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9522,7 +9531,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9601,7 +9610,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9680,7 +9689,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9761,7 +9770,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9842,7 +9851,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9921,7 +9930,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -10000,7 +10009,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10079,7 +10088,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10158,7 +10167,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10237,7 +10246,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10318,7 +10327,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10399,7 +10408,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10478,7 +10487,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10557,7 +10566,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10636,7 +10645,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10715,7 +10724,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10794,7 +10803,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10875,7 +10884,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10954,7 +10963,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -11035,7 +11044,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11114,7 +11123,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11193,7 +11202,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11272,7 +11281,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11351,7 +11360,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11430,7 +11439,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11511,7 +11520,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11590,7 +11599,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11669,7 +11678,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11751,7 +11760,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11830,7 +11839,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11909,7 +11918,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -11988,7 +11997,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -12067,7 +12076,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12146,7 +12155,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12225,7 +12234,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12304,7 +12313,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12383,7 +12392,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12462,7 +12471,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12541,7 +12550,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12620,7 +12629,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12699,7 +12708,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12778,7 +12787,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12857,7 +12866,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12936,7 +12945,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -13015,7 +13024,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13094,7 +13103,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13173,7 +13182,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13252,7 +13261,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13331,7 +13340,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13410,7 +13419,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13489,7 +13498,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13568,7 +13577,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13647,7 +13656,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13726,7 +13735,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13805,7 +13814,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13884,7 +13893,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -13963,7 +13972,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -14042,7 +14051,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14121,7 +14130,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14200,7 +14209,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14279,7 +14288,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14360,7 +14369,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14439,7 +14448,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14518,7 +14527,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14597,7 +14606,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14676,7 +14685,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14755,7 +14764,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14836,7 +14845,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14917,7 +14926,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -14996,7 +15005,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -15075,7 +15084,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15154,7 +15163,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15233,7 +15242,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15314,7 +15323,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15393,7 +15402,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15472,7 +15481,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15551,7 +15560,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15630,7 +15639,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15709,7 +15718,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15788,7 +15797,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15867,7 +15876,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15946,7 +15955,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -16025,7 +16034,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16104,7 +16113,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16183,7 +16192,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16264,7 +16273,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16345,7 +16354,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16424,7 +16433,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16503,7 +16512,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16582,7 +16591,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16661,7 +16670,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16740,7 +16749,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16822,7 +16831,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16901,7 +16910,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -16980,7 +16989,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -17059,7 +17068,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17138,7 +17147,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17219,7 +17228,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17300,7 +17309,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17379,7 +17388,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17458,7 +17467,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17537,7 +17546,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17616,7 +17625,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17695,7 +17704,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17774,7 +17783,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17853,7 +17862,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17932,7 +17941,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -18011,7 +18020,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18090,7 +18099,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18171,7 +18180,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18250,7 +18259,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18329,7 +18338,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18408,7 +18417,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18487,7 +18496,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18566,7 +18575,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18645,7 +18654,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18724,7 +18733,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18803,7 +18812,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18882,7 +18891,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -18961,7 +18970,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -19040,7 +19049,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19119,7 +19128,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19198,7 +19207,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19277,7 +19286,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19356,7 +19365,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19435,7 +19444,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19514,7 +19523,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19595,7 +19604,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19674,7 +19683,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19756,7 +19765,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19838,7 +19847,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19917,7 +19926,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -19996,7 +20005,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20077,7 +20086,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20156,7 +20165,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20235,7 +20244,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20314,7 +20323,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20393,7 +20402,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20472,7 +20481,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20553,7 +20562,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20632,7 +20641,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20711,7 +20720,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20792,7 +20801,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20873,7 +20882,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20954,7 +20963,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -21037,7 +21046,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21118,7 +21127,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21199,7 +21208,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21280,7 +21289,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21361,7 +21370,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21442,7 +21451,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21525,7 +21534,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21608,7 +21617,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21691,7 +21700,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21774,7 +21783,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21855,7 +21864,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21936,7 +21945,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -22019,7 +22028,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22098,7 +22107,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22177,7 +22186,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22256,7 +22265,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22335,7 +22344,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22414,7 +22423,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22495,7 +22504,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22574,7 +22583,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22653,7 +22662,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22732,7 +22741,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22811,7 +22820,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22890,7 +22899,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -22971,7 +22980,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -23050,7 +23059,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23129,7 +23138,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23210,7 +23219,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23289,7 +23298,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23368,7 +23377,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23447,7 +23456,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23526,7 +23535,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23605,7 +23614,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23684,7 +23693,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23763,7 +23772,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23842,7 +23851,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23923,7 +23932,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -24002,7 +24011,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24081,7 +24090,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24160,7 +24169,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24239,7 +24248,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24318,7 +24327,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24397,7 +24406,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24476,7 +24485,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24555,7 +24564,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24634,7 +24643,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24713,7 +24722,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24792,7 +24801,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24871,7 +24880,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24953,7 +24962,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -25032,7 +25041,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25111,7 +25120,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25190,7 +25199,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25269,7 +25278,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25348,7 +25357,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25427,7 +25436,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25506,7 +25515,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25585,7 +25594,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25664,7 +25673,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25743,7 +25752,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25822,7 +25831,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25901,7 +25910,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -25980,7 +25989,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -26059,7 +26068,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26138,7 +26147,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26217,7 +26226,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26296,7 +26305,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26375,7 +26384,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26454,7 +26463,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26533,7 +26542,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26612,7 +26621,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26691,7 +26700,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26770,7 +26779,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26849,7 +26858,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26928,7 +26937,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -27007,7 +27016,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27086,7 +27095,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27165,7 +27174,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27244,7 +27253,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27323,7 +27332,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27402,7 +27411,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27481,7 +27490,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27560,7 +27569,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27639,7 +27648,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27718,7 +27727,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27797,7 +27806,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27876,7 +27885,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -27955,7 +27964,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -28034,7 +28043,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28113,7 +28122,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28192,7 +28201,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28271,7 +28280,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28350,7 +28359,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28429,7 +28438,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28508,7 +28517,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28587,7 +28596,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28666,7 +28675,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28745,7 +28754,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28824,7 +28833,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28903,7 +28912,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -28982,7 +28991,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -29061,7 +29070,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29140,7 +29149,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29219,7 +29228,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29298,7 +29307,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29377,7 +29386,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29456,7 +29465,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:50</v>
+        <v>01:55</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Refactor API client components: Update BaseApiClient to use ExtendedRequestConfig, modify BatchRequestManager to streamline request handling, enhance PremiumPlanService with improved error messaging, and simplify SubscriptionService response structure. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0A94D47-EB38-414E-9E37-725EAC88550C}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43CEE80F-D70D-4CBE-81AD-2823A128AD66}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1547" uniqueCount="924">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1548" uniqueCount="925">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5374,6 +5374,10 @@
   </si>
   <si>
     <t>Found 56 errors in 14 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 47 errors in 11 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6146,7 +6150,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D29"/>
+  <dimension ref="B2:D30"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6299,6 +6303,11 @@
     <row r="29" spans="3:3">
       <c r="C29" t="s">
         <v>923</v>
+      </c>
+    </row>
+    <row r="30" spans="3:3">
+      <c r="C30" t="s">
+        <v>924</v>
       </c>
     </row>
   </sheetData>
@@ -6465,7 +6474,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6476,7 +6485,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>01:57</v>
+        <v>02:05</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6675,7 +6684,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6754,7 +6763,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6833,7 +6842,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6912,7 +6921,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -6991,7 +7000,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -7070,7 +7079,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7149,7 +7158,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7228,7 +7237,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7307,7 +7316,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7386,7 +7395,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7465,7 +7474,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7544,7 +7553,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7623,7 +7632,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7702,7 +7711,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7781,7 +7790,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7860,7 +7869,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7939,7 +7948,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -8018,7 +8027,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8097,7 +8106,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8176,7 +8185,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8255,7 +8264,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8334,7 +8343,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8413,7 +8422,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8492,7 +8501,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8571,7 +8580,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8652,7 +8661,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8733,7 +8742,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8814,7 +8823,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8893,7 +8902,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -8972,7 +8981,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -9051,7 +9060,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9132,7 +9141,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9213,7 +9222,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9294,7 +9303,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9373,7 +9382,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9452,7 +9461,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9531,7 +9540,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9610,7 +9619,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9689,7 +9698,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9770,7 +9779,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9851,7 +9860,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9930,7 +9939,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -10009,7 +10018,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10088,7 +10097,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10167,7 +10176,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10246,7 +10255,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10327,7 +10336,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10408,7 +10417,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10487,7 +10496,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10566,7 +10575,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10645,7 +10654,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10724,7 +10733,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10803,7 +10812,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10884,7 +10893,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10963,7 +10972,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -11044,7 +11053,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11123,7 +11132,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11202,7 +11211,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11281,7 +11290,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11360,7 +11369,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11439,7 +11448,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11520,7 +11529,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11599,7 +11608,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11678,7 +11687,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11760,7 +11769,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11839,7 +11848,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11918,7 +11927,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -11997,7 +12006,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -12076,7 +12085,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12155,7 +12164,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12234,7 +12243,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12313,7 +12322,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12392,7 +12401,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12471,7 +12480,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12550,7 +12559,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12629,7 +12638,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12708,7 +12717,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12787,7 +12796,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12866,7 +12875,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12945,7 +12954,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -13024,7 +13033,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13103,7 +13112,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13182,7 +13191,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13261,7 +13270,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13340,7 +13349,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13419,7 +13428,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13498,7 +13507,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13577,7 +13586,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13656,7 +13665,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13735,7 +13744,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13814,7 +13823,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13893,7 +13902,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -13972,7 +13981,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -14051,7 +14060,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14130,7 +14139,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14209,7 +14218,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14288,7 +14297,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14369,7 +14378,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14448,7 +14457,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14527,7 +14536,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14606,7 +14615,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14685,7 +14694,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14764,7 +14773,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14845,7 +14854,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14926,7 +14935,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -15005,7 +15014,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -15084,7 +15093,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15163,7 +15172,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15242,7 +15251,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15323,7 +15332,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15402,7 +15411,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15481,7 +15490,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15560,7 +15569,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15639,7 +15648,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15718,7 +15727,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15797,7 +15806,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15876,7 +15885,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15955,7 +15964,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -16034,7 +16043,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16113,7 +16122,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16192,7 +16201,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16273,7 +16282,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16354,7 +16363,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16433,7 +16442,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16512,7 +16521,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16591,7 +16600,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16670,7 +16679,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16749,7 +16758,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16831,7 +16840,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16910,7 +16919,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -16989,7 +16998,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -17068,7 +17077,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17147,7 +17156,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17228,7 +17237,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17309,7 +17318,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17388,7 +17397,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17467,7 +17476,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17546,7 +17555,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17625,7 +17634,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17704,7 +17713,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17783,7 +17792,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17862,7 +17871,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17941,7 +17950,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -18020,7 +18029,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18099,7 +18108,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18180,7 +18189,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18259,7 +18268,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18338,7 +18347,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18417,7 +18426,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18496,7 +18505,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18575,7 +18584,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18654,7 +18663,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18733,7 +18742,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18812,7 +18821,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18891,7 +18900,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -18970,7 +18979,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -19049,7 +19058,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19128,7 +19137,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19207,7 +19216,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19286,7 +19295,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19365,7 +19374,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19444,7 +19453,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19523,7 +19532,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19604,7 +19613,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19683,7 +19692,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19765,7 +19774,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19847,7 +19856,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19926,7 +19935,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -20005,7 +20014,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20086,7 +20095,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20165,7 +20174,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20244,7 +20253,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20323,7 +20332,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20402,7 +20411,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20481,7 +20490,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20562,7 +20571,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20641,7 +20650,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20720,7 +20729,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20801,7 +20810,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20882,7 +20891,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20963,7 +20972,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -21046,7 +21055,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21127,7 +21136,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21208,7 +21217,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21289,7 +21298,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21370,7 +21379,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21451,7 +21460,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21534,7 +21543,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21617,7 +21626,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21700,7 +21709,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21783,7 +21792,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21864,7 +21873,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21945,7 +21954,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -22028,7 +22037,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22107,7 +22116,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22186,7 +22195,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22265,7 +22274,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22344,7 +22353,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22423,7 +22432,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22504,7 +22513,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22583,7 +22592,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22662,7 +22671,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22741,7 +22750,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22820,7 +22829,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22899,7 +22908,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -22980,7 +22989,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -23059,7 +23068,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23138,7 +23147,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23219,7 +23228,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23298,7 +23307,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23377,7 +23386,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23456,7 +23465,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23535,7 +23544,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23614,7 +23623,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23693,7 +23702,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23772,7 +23781,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23851,7 +23860,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23932,7 +23941,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -24011,7 +24020,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24090,7 +24099,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24169,7 +24178,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24248,7 +24257,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24327,7 +24336,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24406,7 +24415,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24485,7 +24494,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24564,7 +24573,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24643,7 +24652,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24722,7 +24731,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24801,7 +24810,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24880,7 +24889,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24962,7 +24971,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -25041,7 +25050,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25120,7 +25129,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25199,7 +25208,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25278,7 +25287,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25357,7 +25366,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25436,7 +25445,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25515,7 +25524,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25594,7 +25603,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25673,7 +25682,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25752,7 +25761,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25831,7 +25840,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25910,7 +25919,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -25989,7 +25998,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -26068,7 +26077,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26147,7 +26156,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26226,7 +26235,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26305,7 +26314,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26384,7 +26393,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26463,7 +26472,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26542,7 +26551,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26621,7 +26630,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26700,7 +26709,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26779,7 +26788,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26858,7 +26867,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26937,7 +26946,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -27016,7 +27025,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27095,7 +27104,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27174,7 +27183,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27253,7 +27262,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27332,7 +27341,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27411,7 +27420,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27490,7 +27499,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27569,7 +27578,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27648,7 +27657,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27727,7 +27736,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27806,7 +27815,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27885,7 +27894,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -27964,7 +27973,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -28043,7 +28052,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28122,7 +28131,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28201,7 +28210,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28280,7 +28289,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28359,7 +28368,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28438,7 +28447,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28517,7 +28526,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28596,7 +28605,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28675,7 +28684,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28754,7 +28763,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28833,7 +28842,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28912,7 +28921,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -28991,7 +29000,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -29070,7 +29079,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29149,7 +29158,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29228,7 +29237,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29307,7 +29316,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29386,7 +29395,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29465,7 +29474,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>01:55</v>
+        <v>02:05</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Refactor PremiumPlanService and SubscriptionService: Improve error messaging in PremiumPlanService for better clarity, simplify response handling in SubscriptionService, and enhance type safety in analytics functions. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43CEE80F-D70D-4CBE-81AD-2823A128AD66}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD0F5074-14FB-40EA-8A06-30C32E352E83}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1548" uniqueCount="925">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1549" uniqueCount="926">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5378,6 +5378,10 @@
   </si>
   <si>
     <t>Found 47 errors in 11 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 36 errors in 8 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6150,7 +6154,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D30"/>
+  <dimension ref="B2:D31"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6308,6 +6312,11 @@
     <row r="30" spans="3:3">
       <c r="C30" t="s">
         <v>924</v>
+      </c>
+    </row>
+    <row r="31" spans="3:3">
+      <c r="C31" t="s">
+        <v>925</v>
       </c>
     </row>
   </sheetData>
@@ -6474,7 +6483,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6485,7 +6494,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6684,7 +6693,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6763,7 +6772,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6842,7 +6851,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6921,7 +6930,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -7000,7 +7009,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -7079,7 +7088,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7158,7 +7167,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7237,7 +7246,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7316,7 +7325,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7395,7 +7404,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7474,7 +7483,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7553,7 +7562,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7632,7 +7641,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7711,7 +7720,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7790,7 +7799,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7869,7 +7878,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7948,7 +7957,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -8027,7 +8036,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8106,7 +8115,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8185,7 +8194,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8264,7 +8273,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8343,7 +8352,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8422,7 +8431,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8501,7 +8510,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8580,7 +8589,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8661,7 +8670,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8742,7 +8751,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8823,7 +8832,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8902,7 +8911,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -8981,7 +8990,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -9060,7 +9069,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9141,7 +9150,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9222,7 +9231,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9303,7 +9312,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9382,7 +9391,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9461,7 +9470,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9540,7 +9549,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9619,7 +9628,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9698,7 +9707,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9779,7 +9788,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9860,7 +9869,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9939,7 +9948,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -10018,7 +10027,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10097,7 +10106,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10176,7 +10185,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10255,7 +10264,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10336,7 +10345,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10417,7 +10426,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10496,7 +10505,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10575,7 +10584,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10654,7 +10663,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10733,7 +10742,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10812,7 +10821,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10893,7 +10902,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10972,7 +10981,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -11053,7 +11062,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11132,7 +11141,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11211,7 +11220,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11290,7 +11299,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11369,7 +11378,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11448,7 +11457,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11529,7 +11538,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11608,7 +11617,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11687,7 +11696,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11769,7 +11778,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11848,7 +11857,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11927,7 +11936,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -12006,7 +12015,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -12085,7 +12094,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12164,7 +12173,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12243,7 +12252,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12322,7 +12331,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12401,7 +12410,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12480,7 +12489,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12559,7 +12568,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12638,7 +12647,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12717,7 +12726,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12796,7 +12805,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12875,7 +12884,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12954,7 +12963,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -13033,7 +13042,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13112,7 +13121,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13191,7 +13200,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13270,7 +13279,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13349,7 +13358,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13428,7 +13437,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13507,7 +13516,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13586,7 +13595,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13665,7 +13674,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13744,7 +13753,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13823,7 +13832,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13902,7 +13911,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -13981,7 +13990,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -14060,7 +14069,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14139,7 +14148,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14218,7 +14227,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14297,7 +14306,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14378,7 +14387,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14457,7 +14466,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14536,7 +14545,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14615,7 +14624,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14694,7 +14703,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14773,7 +14782,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14854,7 +14863,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14935,7 +14944,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -15014,7 +15023,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -15093,7 +15102,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15172,7 +15181,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15251,7 +15260,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15332,7 +15341,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15411,7 +15420,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15490,7 +15499,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15569,7 +15578,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15648,7 +15657,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15727,7 +15736,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15806,7 +15815,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15885,7 +15894,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15964,7 +15973,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -16043,7 +16052,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16122,7 +16131,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16201,7 +16210,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16282,7 +16291,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16363,7 +16372,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16442,7 +16451,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16521,7 +16530,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16600,7 +16609,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16679,7 +16688,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16758,7 +16767,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16840,7 +16849,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16919,7 +16928,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -16998,7 +17007,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -17077,7 +17086,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17156,7 +17165,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17237,7 +17246,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17318,7 +17327,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17397,7 +17406,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17476,7 +17485,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17555,7 +17564,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17634,7 +17643,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17713,7 +17722,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17792,7 +17801,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17871,7 +17880,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17950,7 +17959,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -18029,7 +18038,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18108,7 +18117,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18189,7 +18198,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18268,7 +18277,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18347,7 +18356,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18426,7 +18435,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18505,7 +18514,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18584,7 +18593,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18663,7 +18672,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18742,7 +18751,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18821,7 +18830,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18900,7 +18909,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -18979,7 +18988,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -19058,7 +19067,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19137,7 +19146,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19216,7 +19225,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19295,7 +19304,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19374,7 +19383,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19453,7 +19462,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19532,7 +19541,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19613,7 +19622,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19692,7 +19701,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19774,7 +19783,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19856,7 +19865,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19935,7 +19944,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -20014,7 +20023,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20095,7 +20104,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20174,7 +20183,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20253,7 +20262,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20332,7 +20341,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20411,7 +20420,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20490,7 +20499,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20571,7 +20580,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20650,7 +20659,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20729,7 +20738,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20810,7 +20819,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20891,7 +20900,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20972,7 +20981,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -21055,7 +21064,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21136,7 +21145,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21217,7 +21226,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21298,7 +21307,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21379,7 +21388,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21460,7 +21469,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21543,7 +21552,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21626,7 +21635,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21709,7 +21718,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21792,7 +21801,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21873,7 +21882,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21954,7 +21963,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -22037,7 +22046,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22116,7 +22125,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22195,7 +22204,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22274,7 +22283,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22353,7 +22362,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22432,7 +22441,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22513,7 +22522,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22592,7 +22601,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22671,7 +22680,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22750,7 +22759,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22829,7 +22838,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22908,7 +22917,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -22989,7 +22998,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -23068,7 +23077,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23147,7 +23156,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23228,7 +23237,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23307,7 +23316,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23386,7 +23395,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23465,7 +23474,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23544,7 +23553,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23623,7 +23632,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23702,7 +23711,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23781,7 +23790,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23860,7 +23869,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23941,7 +23950,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -24020,7 +24029,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24099,7 +24108,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24178,7 +24187,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24257,7 +24266,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24336,7 +24345,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24415,7 +24424,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24494,7 +24503,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24573,7 +24582,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24652,7 +24661,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24731,7 +24740,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24810,7 +24819,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24889,7 +24898,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24971,7 +24980,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -25050,7 +25059,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25129,7 +25138,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25208,7 +25217,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25287,7 +25296,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25366,7 +25375,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25445,7 +25454,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25524,7 +25533,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25603,7 +25612,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25682,7 +25691,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25761,7 +25770,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25840,7 +25849,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25919,7 +25928,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -25998,7 +26007,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -26077,7 +26086,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26156,7 +26165,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26235,7 +26244,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26314,7 +26323,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26393,7 +26402,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26472,7 +26481,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26551,7 +26560,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26630,7 +26639,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26709,7 +26718,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26788,7 +26797,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26867,7 +26876,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26946,7 +26955,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -27025,7 +27034,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27104,7 +27113,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27183,7 +27192,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27262,7 +27271,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27341,7 +27350,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27420,7 +27429,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27499,7 +27508,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27578,7 +27587,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27657,7 +27666,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27736,7 +27745,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27815,7 +27824,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27894,7 +27903,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -27973,7 +27982,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -28052,7 +28061,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28131,7 +28140,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28210,7 +28219,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28289,7 +28298,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28368,7 +28377,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28447,7 +28456,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28526,7 +28535,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28605,7 +28614,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28684,7 +28693,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28763,7 +28772,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28842,7 +28851,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28921,7 +28930,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -29000,7 +29009,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -29079,7 +29088,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29158,7 +29167,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29237,7 +29246,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29316,7 +29325,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29395,7 +29404,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29474,7 +29483,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:05</v>
+        <v>02:10</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Refactor SubscriptionService and ApiClient: Simplify response handling in SubscriptionService, enhance error response structure, and improve request configuration in ApiClient. Update analytics functions for better type safety and add billingDate property to Subscription interface. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD0F5074-14FB-40EA-8A06-30C32E352E83}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09F1C063-48DE-46FA-82A3-7B9297622148}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1549" uniqueCount="926">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1550" uniqueCount="927">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5382,6 +5382,10 @@
   </si>
   <si>
     <t>Found 36 errors in 8 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 34 errors in 9 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6154,7 +6158,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D31"/>
+  <dimension ref="B2:D32"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6317,6 +6321,11 @@
     <row r="31" spans="3:3">
       <c r="C31" t="s">
         <v>925</v>
+      </c>
+    </row>
+    <row r="32" spans="3:3">
+      <c r="C32" t="s">
+        <v>926</v>
       </c>
     </row>
   </sheetData>
@@ -6483,7 +6492,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6494,7 +6503,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6693,7 +6702,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6772,7 +6781,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6851,7 +6860,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6930,7 +6939,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -7009,7 +7018,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -7088,7 +7097,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7167,7 +7176,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7246,7 +7255,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7325,7 +7334,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7404,7 +7413,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7483,7 +7492,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7562,7 +7571,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7641,7 +7650,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7720,7 +7729,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7799,7 +7808,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7878,7 +7887,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7957,7 +7966,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -8036,7 +8045,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8115,7 +8124,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8194,7 +8203,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8273,7 +8282,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8352,7 +8361,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8431,7 +8440,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8510,7 +8519,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8589,7 +8598,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8670,7 +8679,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8751,7 +8760,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8832,7 +8841,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8911,7 +8920,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -8990,7 +8999,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -9069,7 +9078,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9150,7 +9159,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9231,7 +9240,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9312,7 +9321,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9391,7 +9400,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9470,7 +9479,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9549,7 +9558,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9628,7 +9637,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9707,7 +9716,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9788,7 +9797,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9869,7 +9878,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9948,7 +9957,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -10027,7 +10036,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10106,7 +10115,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10185,7 +10194,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10264,7 +10273,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10345,7 +10354,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10426,7 +10435,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10505,7 +10514,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10584,7 +10593,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10663,7 +10672,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10742,7 +10751,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10821,7 +10830,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10902,7 +10911,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10981,7 +10990,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -11062,7 +11071,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11141,7 +11150,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11220,7 +11229,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11299,7 +11308,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11378,7 +11387,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11457,7 +11466,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11538,7 +11547,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11617,7 +11626,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11696,7 +11705,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11778,7 +11787,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11857,7 +11866,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11936,7 +11945,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -12015,7 +12024,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -12094,7 +12103,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12173,7 +12182,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12252,7 +12261,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12331,7 +12340,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12410,7 +12419,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12489,7 +12498,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12568,7 +12577,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12647,7 +12656,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12726,7 +12735,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12805,7 +12814,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12884,7 +12893,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12963,7 +12972,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -13042,7 +13051,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13121,7 +13130,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13200,7 +13209,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13279,7 +13288,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13358,7 +13367,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13437,7 +13446,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13516,7 +13525,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13595,7 +13604,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13674,7 +13683,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13753,7 +13762,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13832,7 +13841,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13911,7 +13920,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -13990,7 +13999,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -14069,7 +14078,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14148,7 +14157,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14227,7 +14236,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14306,7 +14315,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14387,7 +14396,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14466,7 +14475,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14545,7 +14554,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14624,7 +14633,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14703,7 +14712,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14782,7 +14791,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14863,7 +14872,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14944,7 +14953,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -15023,7 +15032,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -15102,7 +15111,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15181,7 +15190,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15260,7 +15269,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15341,7 +15350,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15420,7 +15429,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15499,7 +15508,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15578,7 +15587,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15657,7 +15666,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15736,7 +15745,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15815,7 +15824,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15894,7 +15903,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15973,7 +15982,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -16052,7 +16061,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16131,7 +16140,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16210,7 +16219,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16291,7 +16300,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16372,7 +16381,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16451,7 +16460,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16530,7 +16539,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16609,7 +16618,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16688,7 +16697,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16767,7 +16776,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16849,7 +16858,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16928,7 +16937,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -17007,7 +17016,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -17086,7 +17095,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17165,7 +17174,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17246,7 +17255,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17327,7 +17336,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17406,7 +17415,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17485,7 +17494,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17564,7 +17573,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17643,7 +17652,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17722,7 +17731,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17801,7 +17810,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17880,7 +17889,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17959,7 +17968,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -18038,7 +18047,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18117,7 +18126,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18198,7 +18207,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18277,7 +18286,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18356,7 +18365,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18435,7 +18444,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18514,7 +18523,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18593,7 +18602,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18672,7 +18681,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18751,7 +18760,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18830,7 +18839,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18909,7 +18918,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -18988,7 +18997,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -19067,7 +19076,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19146,7 +19155,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19225,7 +19234,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19304,7 +19313,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19383,7 +19392,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19462,7 +19471,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19541,7 +19550,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19622,7 +19631,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19701,7 +19710,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19783,7 +19792,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19865,7 +19874,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19944,7 +19953,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -20023,7 +20032,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20104,7 +20113,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20183,7 +20192,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20262,7 +20271,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20341,7 +20350,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20420,7 +20429,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20499,7 +20508,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20580,7 +20589,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20659,7 +20668,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20738,7 +20747,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20819,7 +20828,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20900,7 +20909,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20981,7 +20990,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -21064,7 +21073,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21145,7 +21154,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21226,7 +21235,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21307,7 +21316,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21388,7 +21397,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21469,7 +21478,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21552,7 +21561,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21635,7 +21644,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21718,7 +21727,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21801,7 +21810,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21882,7 +21891,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21963,7 +21972,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -22046,7 +22055,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22125,7 +22134,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22204,7 +22213,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22283,7 +22292,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22362,7 +22371,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22441,7 +22450,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22522,7 +22531,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22601,7 +22610,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22680,7 +22689,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22759,7 +22768,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22838,7 +22847,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22917,7 +22926,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -22998,7 +23007,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -23077,7 +23086,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23156,7 +23165,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23237,7 +23246,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23316,7 +23325,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23395,7 +23404,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23474,7 +23483,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23553,7 +23562,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23632,7 +23641,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23711,7 +23720,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23790,7 +23799,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23869,7 +23878,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23950,7 +23959,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -24029,7 +24038,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24108,7 +24117,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24187,7 +24196,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24266,7 +24275,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24345,7 +24354,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24424,7 +24433,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24503,7 +24512,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24582,7 +24591,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24661,7 +24670,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24740,7 +24749,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24819,7 +24828,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24898,7 +24907,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24980,7 +24989,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -25059,7 +25068,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25138,7 +25147,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25217,7 +25226,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25296,7 +25305,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25375,7 +25384,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25454,7 +25463,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25533,7 +25542,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25612,7 +25621,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25691,7 +25700,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25770,7 +25779,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25849,7 +25858,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25928,7 +25937,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -26007,7 +26016,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -26086,7 +26095,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26165,7 +26174,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26244,7 +26253,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26323,7 +26332,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26402,7 +26411,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26481,7 +26490,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26560,7 +26569,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26639,7 +26648,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26718,7 +26727,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26797,7 +26806,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26876,7 +26885,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26955,7 +26964,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -27034,7 +27043,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27113,7 +27122,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27192,7 +27201,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27271,7 +27280,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27350,7 +27359,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27429,7 +27438,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27508,7 +27517,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27587,7 +27596,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27666,7 +27675,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27745,7 +27754,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27824,7 +27833,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27903,7 +27912,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -27982,7 +27991,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -28061,7 +28070,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28140,7 +28149,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28219,7 +28228,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28298,7 +28307,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28377,7 +28386,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28456,7 +28465,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28535,7 +28544,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28614,7 +28623,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28693,7 +28702,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28772,7 +28781,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28851,7 +28860,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28930,7 +28939,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -29009,7 +29018,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -29088,7 +29097,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29167,7 +29176,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29246,7 +29255,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29325,7 +29334,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29404,7 +29413,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29483,7 +29492,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:10</v>
+        <v>02:15</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Refactor API and service components: Simplify request handling in PremiumPlanService and SubscriptionService, enhance error response structure in ApiClient, and improve type safety in SubscriptionManagementPage. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09F1C063-48DE-46FA-82A3-7B9297622148}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA1CAEA5-E758-4272-A02F-8C2CC5F0D64B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1550" uniqueCount="927">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1551" uniqueCount="928">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5386,6 +5386,10 @@
   </si>
   <si>
     <t>Found 34 errors in 9 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 24 errors in 8 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6158,7 +6162,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D32"/>
+  <dimension ref="B2:D33"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6326,6 +6330,11 @@
     <row r="32" spans="3:3">
       <c r="C32" t="s">
         <v>926</v>
+      </c>
+    </row>
+    <row r="33" spans="3:3">
+      <c r="C33" t="s">
+        <v>927</v>
       </c>
     </row>
   </sheetData>
@@ -6503,7 +6512,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>02:15</v>
+        <v>02:19</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">

</xml_diff>

<commit_message>
Update type definition for unregisteredMonths in RegistrationReminderCard component to improve type safety. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA1CAEA5-E758-4272-A02F-8C2CC5F0D64B}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89CC501B-06AB-4281-BEA1-7A52FD14E733}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1551" uniqueCount="928">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="929">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -5390,6 +5390,10 @@
   </si>
   <si>
     <t>Found 24 errors in 8 files.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Found 7 errors in 3 files.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6162,7 +6166,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D33"/>
+  <dimension ref="B2:D34"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6335,6 +6339,11 @@
     <row r="33" spans="3:3">
       <c r="C33" t="s">
         <v>927</v>
+      </c>
+    </row>
+    <row r="34" spans="3:3">
+      <c r="C34" t="s">
+        <v>928</v>
       </c>
     </row>
   </sheetData>
@@ -6501,7 +6510,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6512,7 +6521,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>02:19</v>
+        <v>02:22</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6711,7 +6720,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6790,7 +6799,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6869,7 +6878,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6948,7 +6957,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -7027,7 +7036,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -7106,7 +7115,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7185,7 +7194,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7264,7 +7273,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7343,7 +7352,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7422,7 +7431,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7501,7 +7510,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7580,7 +7589,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7659,7 +7668,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7738,7 +7747,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7817,7 +7826,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7896,7 +7905,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7975,7 +7984,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -8054,7 +8063,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8133,7 +8142,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8212,7 +8221,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8291,7 +8300,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8370,7 +8379,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8449,7 +8458,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8528,7 +8537,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8607,7 +8616,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8688,7 +8697,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8769,7 +8778,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8850,7 +8859,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8929,7 +8938,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -9008,7 +9017,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -9087,7 +9096,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9168,7 +9177,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9249,7 +9258,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9330,7 +9339,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9409,7 +9418,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9488,7 +9497,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9567,7 +9576,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9646,7 +9655,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9725,7 +9734,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9806,7 +9815,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9887,7 +9896,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9966,7 +9975,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -10045,7 +10054,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10124,7 +10133,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10203,7 +10212,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10282,7 +10291,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10363,7 +10372,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10444,7 +10453,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10523,7 +10532,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10602,7 +10611,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10681,7 +10690,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10760,7 +10769,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10839,7 +10848,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10920,7 +10929,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -10999,7 +11008,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -11080,7 +11089,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11159,7 +11168,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11238,7 +11247,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11317,7 +11326,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11396,7 +11405,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11475,7 +11484,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11556,7 +11565,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11635,7 +11644,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11714,7 +11723,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11796,7 +11805,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11875,7 +11884,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11954,7 +11963,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -12033,7 +12042,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -12112,7 +12121,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12191,7 +12200,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12270,7 +12279,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12349,7 +12358,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12428,7 +12437,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12507,7 +12516,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12586,7 +12595,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12665,7 +12674,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12744,7 +12753,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12823,7 +12832,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12902,7 +12911,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12981,7 +12990,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -13060,7 +13069,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13139,7 +13148,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13218,7 +13227,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13297,7 +13306,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13376,7 +13385,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13455,7 +13464,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13534,7 +13543,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13613,7 +13622,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13692,7 +13701,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13771,7 +13780,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13850,7 +13859,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13929,7 +13938,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -14008,7 +14017,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -14087,7 +14096,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14166,7 +14175,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14245,7 +14254,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14324,7 +14333,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14405,7 +14414,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14484,7 +14493,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14563,7 +14572,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14642,7 +14651,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14721,7 +14730,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14800,7 +14809,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14881,7 +14890,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14962,7 +14971,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -15041,7 +15050,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -15120,7 +15129,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15199,7 +15208,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15278,7 +15287,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15359,7 +15368,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15438,7 +15447,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15517,7 +15526,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15596,7 +15605,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15675,7 +15684,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15754,7 +15763,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15833,7 +15842,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15912,7 +15921,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -15991,7 +16000,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -16070,7 +16079,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16149,7 +16158,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16228,7 +16237,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16309,7 +16318,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16390,7 +16399,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16469,7 +16478,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16548,7 +16557,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16627,7 +16636,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16706,7 +16715,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16785,7 +16794,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16867,7 +16876,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16946,7 +16955,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -17025,7 +17034,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -17104,7 +17113,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17183,7 +17192,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17264,7 +17273,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17345,7 +17354,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17424,7 +17433,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17503,7 +17512,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17582,7 +17591,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17661,7 +17670,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17740,7 +17749,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17819,7 +17828,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17898,7 +17907,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17977,7 +17986,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -18056,7 +18065,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18135,7 +18144,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18216,7 +18225,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18295,7 +18304,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18374,7 +18383,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18453,7 +18462,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18532,7 +18541,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18611,7 +18620,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18690,7 +18699,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18769,7 +18778,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18848,7 +18857,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18927,7 +18936,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -19006,7 +19015,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -19085,7 +19094,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19164,7 +19173,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19243,7 +19252,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19322,7 +19331,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19401,7 +19410,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19480,7 +19489,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19559,7 +19568,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19640,7 +19649,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19719,7 +19728,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19801,7 +19810,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19883,7 +19892,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19962,7 +19971,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -20041,7 +20050,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20122,7 +20131,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20201,7 +20210,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20280,7 +20289,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20359,7 +20368,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20438,7 +20447,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20517,7 +20526,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20598,7 +20607,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20677,7 +20686,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20756,7 +20765,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20837,7 +20846,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20918,7 +20927,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -20999,7 +21008,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -21082,7 +21091,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21163,7 +21172,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21244,7 +21253,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21325,7 +21334,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21406,7 +21415,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21487,7 +21496,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21570,7 +21579,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21653,7 +21662,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21736,7 +21745,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21819,7 +21828,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21900,7 +21909,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21981,7 +21990,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -22064,7 +22073,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22143,7 +22152,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22222,7 +22231,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22301,7 +22310,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22380,7 +22389,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22459,7 +22468,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22540,7 +22549,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22619,7 +22628,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22698,7 +22707,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22777,7 +22786,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22856,7 +22865,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22935,7 +22944,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -23016,7 +23025,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -23095,7 +23104,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23174,7 +23183,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23255,7 +23264,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23334,7 +23343,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23413,7 +23422,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23492,7 +23501,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23571,7 +23580,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23650,7 +23659,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23729,7 +23738,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23808,7 +23817,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23887,7 +23896,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23968,7 +23977,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -24047,7 +24056,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24126,7 +24135,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24205,7 +24214,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24284,7 +24293,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24363,7 +24372,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24442,7 +24451,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24521,7 +24530,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24600,7 +24609,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24679,7 +24688,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24758,7 +24767,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24837,7 +24846,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24916,7 +24925,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -24998,7 +25007,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -25077,7 +25086,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25156,7 +25165,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25235,7 +25244,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25314,7 +25323,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25393,7 +25402,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25472,7 +25481,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25551,7 +25560,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25630,7 +25639,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25709,7 +25718,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25788,7 +25797,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25867,7 +25876,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25946,7 +25955,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -26025,7 +26034,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -26104,7 +26113,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26183,7 +26192,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26262,7 +26271,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26341,7 +26350,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26420,7 +26429,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26499,7 +26508,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26578,7 +26587,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26657,7 +26666,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26736,7 +26745,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26815,7 +26824,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26894,7 +26903,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26973,7 +26982,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -27052,7 +27061,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27131,7 +27140,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27210,7 +27219,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27289,7 +27298,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27368,7 +27377,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27447,7 +27456,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27526,7 +27535,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27605,7 +27614,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27684,7 +27693,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27763,7 +27772,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27842,7 +27851,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27921,7 +27930,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -28000,7 +28009,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -28079,7 +28088,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28158,7 +28167,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28237,7 +28246,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28316,7 +28325,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28395,7 +28404,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28474,7 +28483,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28553,7 +28562,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28632,7 +28641,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28711,7 +28720,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28790,7 +28799,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28869,7 +28878,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28948,7 +28957,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -29027,7 +29036,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -29106,7 +29115,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29185,7 +29194,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29264,7 +29273,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29343,7 +29352,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29422,7 +29431,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29501,7 +29510,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:15</v>
+        <v>02:20</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Refactor PremiumPlanService and PremiumPromotion components: Simplify error message handling in PremiumPlanService, enhance data loading in PremiumPromotion with async useEffect, and improve type safety in SubscriptionManagementPage. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89CC501B-06AB-4281-BEA1-7A52FD14E733}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F3E0FBC-1262-4039-B607-4C53D5B1F725}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="929">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1553" uniqueCount="929">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -6166,7 +6166,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083174DA-A42C-4F9C-978E-61AEAAD9DDFF}">
-  <dimension ref="B2:D34"/>
+  <dimension ref="B2:D35"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -6343,6 +6343,11 @@
     </row>
     <row r="34" spans="3:3">
       <c r="C34" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="35" spans="3:3">
+      <c r="C35" t="s">
         <v>928</v>
       </c>
     </row>
@@ -6510,7 +6515,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6521,7 +6526,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>02:22</v>
+        <v>02:25</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6720,7 +6725,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6799,7 +6804,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6878,7 +6883,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6957,7 +6962,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -7036,7 +7041,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -7115,7 +7120,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7194,7 +7199,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7273,7 +7278,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7352,7 +7357,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7431,7 +7436,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7510,7 +7515,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7589,7 +7594,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7668,7 +7673,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7747,7 +7752,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7826,7 +7831,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7905,7 +7910,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7984,7 +7989,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -8063,7 +8068,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8142,7 +8147,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8221,7 +8226,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8300,7 +8305,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8379,7 +8384,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8458,7 +8463,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8537,7 +8542,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8616,7 +8621,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8697,7 +8702,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8778,7 +8783,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8859,7 +8864,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8938,7 +8943,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -9017,7 +9022,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -9096,7 +9101,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9177,7 +9182,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9258,7 +9263,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9339,7 +9344,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9418,7 +9423,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9497,7 +9502,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9576,7 +9581,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9655,7 +9660,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9734,7 +9739,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9815,7 +9820,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9896,7 +9901,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9975,7 +9980,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -10054,7 +10059,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10133,7 +10138,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10212,7 +10217,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10291,7 +10296,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10372,7 +10377,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10453,7 +10458,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10532,7 +10537,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10611,7 +10616,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10690,7 +10695,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10769,7 +10774,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10848,7 +10853,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10929,7 +10934,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -11008,7 +11013,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -11089,7 +11094,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11168,7 +11173,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11247,7 +11252,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11326,7 +11331,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11405,7 +11410,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11484,7 +11489,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11565,7 +11570,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11644,7 +11649,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11723,7 +11728,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11805,7 +11810,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11884,7 +11889,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11963,7 +11968,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -12042,7 +12047,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -12121,7 +12126,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12200,7 +12205,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12279,7 +12284,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12358,7 +12363,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12437,7 +12442,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12516,7 +12521,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12595,7 +12600,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12674,7 +12679,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12753,7 +12758,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12832,7 +12837,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12911,7 +12916,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12990,7 +12995,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -13069,7 +13074,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13148,7 +13153,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13227,7 +13232,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13306,7 +13311,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13385,7 +13390,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13464,7 +13469,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13543,7 +13548,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13622,7 +13627,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13701,7 +13706,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13780,7 +13785,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13859,7 +13864,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13938,7 +13943,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -14017,7 +14022,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -14096,7 +14101,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14175,7 +14180,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14254,7 +14259,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14333,7 +14338,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14414,7 +14419,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14493,7 +14498,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14572,7 +14577,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14651,7 +14656,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14730,7 +14735,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14809,7 +14814,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14890,7 +14895,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14971,7 +14976,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -15050,7 +15055,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -15129,7 +15134,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15208,7 +15213,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15287,7 +15292,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15368,7 +15373,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15447,7 +15452,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15526,7 +15531,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15605,7 +15610,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15684,7 +15689,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15763,7 +15768,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15842,7 +15847,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15921,7 +15926,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -16000,7 +16005,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -16079,7 +16084,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16158,7 +16163,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16237,7 +16242,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16318,7 +16323,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16399,7 +16404,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16478,7 +16483,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16557,7 +16562,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16636,7 +16641,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16715,7 +16720,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16794,7 +16799,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16876,7 +16881,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16955,7 +16960,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -17034,7 +17039,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -17113,7 +17118,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17192,7 +17197,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17273,7 +17278,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17354,7 +17359,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17433,7 +17438,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17512,7 +17517,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17591,7 +17596,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17670,7 +17675,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17749,7 +17754,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17828,7 +17833,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17907,7 +17912,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17986,7 +17991,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -18065,7 +18070,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18144,7 +18149,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18225,7 +18230,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18304,7 +18309,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18383,7 +18388,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18462,7 +18467,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18541,7 +18546,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18620,7 +18625,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18699,7 +18704,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18778,7 +18783,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18857,7 +18862,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18936,7 +18941,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -19015,7 +19020,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -19094,7 +19099,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19173,7 +19178,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19252,7 +19257,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19331,7 +19336,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19410,7 +19415,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19489,7 +19494,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19568,7 +19573,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19649,7 +19654,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19728,7 +19733,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19810,7 +19815,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19892,7 +19897,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19971,7 +19976,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -20050,7 +20055,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20131,7 +20136,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20210,7 +20215,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20289,7 +20294,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20368,7 +20373,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20447,7 +20452,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20526,7 +20531,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20607,7 +20612,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20686,7 +20691,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20765,7 +20770,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20846,7 +20851,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20927,7 +20932,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -21008,7 +21013,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -21091,7 +21096,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21172,7 +21177,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21253,7 +21258,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21334,7 +21339,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21415,7 +21420,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21496,7 +21501,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21579,7 +21584,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21662,7 +21667,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21745,7 +21750,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21828,7 +21833,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21909,7 +21914,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21990,7 +21995,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -22073,7 +22078,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22152,7 +22157,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22231,7 +22236,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22310,7 +22315,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22389,7 +22394,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22468,7 +22473,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22549,7 +22554,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22628,7 +22633,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22707,7 +22712,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22786,7 +22791,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22865,7 +22870,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22944,7 +22949,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -23025,7 +23030,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -23104,7 +23109,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23183,7 +23188,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23264,7 +23269,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23343,7 +23348,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23422,7 +23427,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23501,7 +23506,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23580,7 +23585,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23659,7 +23664,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23738,7 +23743,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23817,7 +23822,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23896,7 +23901,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23977,7 +23982,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -24056,7 +24061,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24135,7 +24140,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24214,7 +24219,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24293,7 +24298,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24372,7 +24377,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24451,7 +24456,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24530,7 +24535,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24609,7 +24614,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24688,7 +24693,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24767,7 +24772,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24846,7 +24851,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24925,7 +24930,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -25007,7 +25012,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -25086,7 +25091,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25165,7 +25170,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25244,7 +25249,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25323,7 +25328,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25402,7 +25407,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25481,7 +25486,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25560,7 +25565,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25639,7 +25644,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25718,7 +25723,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25797,7 +25802,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25876,7 +25881,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25955,7 +25960,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -26034,7 +26039,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -26113,7 +26118,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26192,7 +26197,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26271,7 +26276,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26350,7 +26355,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26429,7 +26434,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26508,7 +26513,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26587,7 +26592,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26666,7 +26671,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26745,7 +26750,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26824,7 +26829,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26903,7 +26908,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26982,7 +26987,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -27061,7 +27066,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27140,7 +27145,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27219,7 +27224,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27298,7 +27303,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27377,7 +27382,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27456,7 +27461,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27535,7 +27540,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27614,7 +27619,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27693,7 +27698,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27772,7 +27777,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27851,7 +27856,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27930,7 +27935,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -28009,7 +28014,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -28088,7 +28093,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28167,7 +28172,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28246,7 +28251,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28325,7 +28330,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28404,7 +28409,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28483,7 +28488,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28562,7 +28567,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28641,7 +28646,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28720,7 +28725,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28799,7 +28804,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28878,7 +28883,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28957,7 +28962,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -29036,7 +29041,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -29115,7 +29120,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29194,7 +29199,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29273,7 +29278,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29352,7 +29357,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29431,7 +29436,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29510,7 +29515,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:20</v>
+        <v>02:25</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Refactor API request handling in BatchRequestManager and ApiManagerHTTPMethods: Enhance type safety, streamline request execution, and introduce optimization features for batch requests. Update Vite-Vercel開発.xlsx file.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c67ec30e06f060f/work/GitHub/work-time-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F3E0FBC-1262-4039-B607-4C53D5B1F725}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{1928CA11-C4AD-40E9-B1C5-143667E830EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23D486BC-AF2B-4C12-BB4A-7472D4A587D8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="よく使うこまんど" sheetId="1" r:id="rId1"/>
@@ -6515,7 +6515,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -6526,7 +6526,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -6725,7 +6725,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -6804,7 +6804,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -6883,7 +6883,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -6962,7 +6962,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -7041,7 +7041,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -7120,7 +7120,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -7199,7 +7199,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -7278,7 +7278,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -7357,7 +7357,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -7436,7 +7436,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -7515,7 +7515,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -7594,7 +7594,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -7673,7 +7673,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -7752,7 +7752,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -7831,7 +7831,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -7910,7 +7910,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -7989,7 +7989,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -8068,7 +8068,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -8147,7 +8147,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -8226,7 +8226,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -8305,7 +8305,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -8384,7 +8384,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -8463,7 +8463,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -8542,7 +8542,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -8621,7 +8621,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -8702,7 +8702,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -8783,7 +8783,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -8864,7 +8864,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -8943,7 +8943,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -9022,7 +9022,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -9101,7 +9101,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -9182,7 +9182,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -9263,7 +9263,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -9344,7 +9344,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -9423,7 +9423,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -9502,7 +9502,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -9581,7 +9581,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -9660,7 +9660,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -9739,7 +9739,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -9820,7 +9820,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -9901,7 +9901,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -9980,7 +9980,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -10059,7 +10059,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -10138,7 +10138,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -10217,7 +10217,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -10296,7 +10296,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -10377,7 +10377,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -10458,7 +10458,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -10537,7 +10537,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -10616,7 +10616,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -10695,7 +10695,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -10774,7 +10774,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -10853,7 +10853,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -10934,7 +10934,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -11013,7 +11013,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -11094,7 +11094,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -11173,7 +11173,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -11252,7 +11252,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -11331,7 +11331,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -11410,7 +11410,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -11489,7 +11489,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -11570,7 +11570,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -11649,7 +11649,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -11728,7 +11728,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -11810,7 +11810,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -11889,7 +11889,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -11968,7 +11968,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -12047,7 +12047,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -12126,7 +12126,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -12205,7 +12205,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -12284,7 +12284,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -12363,7 +12363,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -12442,7 +12442,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -12521,7 +12521,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -12600,7 +12600,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -12679,7 +12679,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -12758,7 +12758,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -12837,7 +12837,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -12916,7 +12916,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -12995,7 +12995,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -13074,7 +13074,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -13153,7 +13153,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -13232,7 +13232,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -13311,7 +13311,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -13390,7 +13390,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -13469,7 +13469,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -13548,7 +13548,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -13627,7 +13627,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -13706,7 +13706,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -13785,7 +13785,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -13864,7 +13864,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -13943,7 +13943,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -14022,7 +14022,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -14101,7 +14101,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -14180,7 +14180,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -14259,7 +14259,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -14338,7 +14338,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -14419,7 +14419,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -14498,7 +14498,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -14577,7 +14577,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -14656,7 +14656,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -14735,7 +14735,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -14814,7 +14814,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -14895,7 +14895,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -14976,7 +14976,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -15055,7 +15055,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -15134,7 +15134,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -15213,7 +15213,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -15292,7 +15292,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -15373,7 +15373,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -15452,7 +15452,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -15531,7 +15531,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -15610,7 +15610,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -15689,7 +15689,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -15768,7 +15768,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -15847,7 +15847,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -15926,7 +15926,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -16005,7 +16005,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -16084,7 +16084,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -16163,7 +16163,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -16242,7 +16242,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -16323,7 +16323,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -16404,7 +16404,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -16483,7 +16483,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -16562,7 +16562,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -16641,7 +16641,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -16720,7 +16720,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -16799,7 +16799,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -16881,7 +16881,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -16960,7 +16960,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -17039,7 +17039,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -17118,7 +17118,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -17197,7 +17197,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -17278,7 +17278,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -17359,7 +17359,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -17438,7 +17438,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -17517,7 +17517,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -17596,7 +17596,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -17675,7 +17675,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -17754,7 +17754,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -17833,7 +17833,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -17912,7 +17912,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -17991,7 +17991,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -18070,7 +18070,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -18149,7 +18149,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -18230,7 +18230,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -18309,7 +18309,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -18388,7 +18388,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -18467,7 +18467,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -18546,7 +18546,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -18625,7 +18625,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -18704,7 +18704,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -18783,7 +18783,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -18862,7 +18862,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -18941,7 +18941,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -19020,7 +19020,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -19099,7 +19099,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -19178,7 +19178,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -19257,7 +19257,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -19336,7 +19336,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -19415,7 +19415,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -19494,7 +19494,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -19573,7 +19573,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -19654,7 +19654,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -19733,7 +19733,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -19815,7 +19815,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -19897,7 +19897,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -19976,7 +19976,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -20055,7 +20055,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -20136,7 +20136,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -20215,7 +20215,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -20294,7 +20294,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -20373,7 +20373,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -20452,7 +20452,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -20531,7 +20531,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -20612,7 +20612,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -20691,7 +20691,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -20770,7 +20770,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -20851,7 +20851,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -20932,7 +20932,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -21013,7 +21013,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -21096,7 +21096,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -21177,7 +21177,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -21258,7 +21258,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -21339,7 +21339,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -21420,7 +21420,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -21501,7 +21501,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -21584,7 +21584,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -21667,7 +21667,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -21750,7 +21750,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -21833,7 +21833,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -21914,7 +21914,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -21995,7 +21995,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -22078,7 +22078,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -22157,7 +22157,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -22236,7 +22236,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -22315,7 +22315,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -22394,7 +22394,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -22473,7 +22473,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -22554,7 +22554,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -22633,7 +22633,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -22712,7 +22712,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -22791,7 +22791,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -22870,7 +22870,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -22949,7 +22949,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -23030,7 +23030,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -23109,7 +23109,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -23188,7 +23188,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -23269,7 +23269,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -23348,7 +23348,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -23427,7 +23427,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -23506,7 +23506,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -23585,7 +23585,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -23664,7 +23664,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -23743,7 +23743,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -23822,7 +23822,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -23901,7 +23901,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -23982,7 +23982,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -24061,7 +24061,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -24140,7 +24140,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -24219,7 +24219,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -24298,7 +24298,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -24377,7 +24377,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -24456,7 +24456,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -24535,7 +24535,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -24614,7 +24614,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -24693,7 +24693,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -24772,7 +24772,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -24851,7 +24851,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -24930,7 +24930,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -25012,7 +25012,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -25091,7 +25091,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -25170,7 +25170,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -25249,7 +25249,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -25328,7 +25328,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -25407,7 +25407,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -25486,7 +25486,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -25565,7 +25565,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -25644,7 +25644,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -25723,7 +25723,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -25802,7 +25802,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -25881,7 +25881,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -25960,7 +25960,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -26039,7 +26039,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -26118,7 +26118,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -26197,7 +26197,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -26276,7 +26276,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -26355,7 +26355,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -26434,7 +26434,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -26513,7 +26513,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -26592,7 +26592,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -26671,7 +26671,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -26750,7 +26750,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -26829,7 +26829,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -26908,7 +26908,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -26987,7 +26987,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -27066,7 +27066,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -27145,7 +27145,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -27224,7 +27224,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -27303,7 +27303,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -27382,7 +27382,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -27461,7 +27461,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -27540,7 +27540,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -27619,7 +27619,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -27698,7 +27698,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -27777,7 +27777,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -27856,7 +27856,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -27935,7 +27935,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -28014,7 +28014,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -28093,7 +28093,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -28172,7 +28172,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -28251,7 +28251,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -28330,7 +28330,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -28409,7 +28409,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -28488,7 +28488,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -28567,7 +28567,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -28646,7 +28646,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -28725,7 +28725,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -28804,7 +28804,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -28883,7 +28883,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -28962,7 +28962,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -29041,7 +29041,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -29120,7 +29120,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -29199,7 +29199,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -29278,7 +29278,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -29357,7 +29357,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -29436,7 +29436,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -29515,7 +29515,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>02:25</v>
+        <v>02:55</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Update DevelopmentBadgeDashboard component by removing unused icon imports for improved performance. Additionally, update the associated Excel file to reflect recent changes.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\work-time-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AD7BDB1-E5EC-451D-AC3E-EADD56B89E47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAFCF071-F655-4E45-8BFA-B74FC39138C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1807" uniqueCount="1156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1814" uniqueCount="1164">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -10887,6 +10887,47 @@
   </si>
   <si>
     <t>https://work-time-tracker-5d9q.vercel.app/bookshelf</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ショップ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://work-time-tracker-5d9q.vercel.app/shop</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://work-time-tracker-5d9q.vercel.app/products</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>商品一覧</t>
+    <rPh sb="0" eb="2">
+      <t>ショウヒン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>イチラン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Twitter</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://work-time-tracker-5d9q.vercel.app/twitter</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://work-time-tracker-5d9q.vercel.app/political-trends</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>政治トレンド</t>
+    <rPh sb="0" eb="2">
+      <t>セイジ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -11685,7 +11726,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{485A7026-3BCD-4330-8EB1-BC125AB72393}">
-  <dimension ref="B2:G23"/>
+  <dimension ref="B2:G26"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
@@ -11894,8 +11935,8 @@
       <c r="D14" s="2" t="s">
         <v>1155</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>1117</v>
+      <c r="E14" s="1">
+        <v>45829</v>
       </c>
     </row>
     <row r="15" spans="2:7">
@@ -11999,8 +12040,8 @@
       <c r="D21" s="2" t="s">
         <v>1152</v>
       </c>
-      <c r="E21" t="s">
-        <v>1117</v>
+      <c r="E21" s="1">
+        <v>45829</v>
       </c>
     </row>
     <row r="22" spans="2:5">
@@ -12022,6 +12063,60 @@
       <c r="B23">
         <f>B22+1</f>
         <v>21</v>
+      </c>
+      <c r="C23" t="s">
+        <v>1156</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="E23" s="1">
+        <v>45829</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5">
+      <c r="B24">
+        <f>B23+1</f>
+        <v>22</v>
+      </c>
+      <c r="C24" t="s">
+        <v>1159</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>1158</v>
+      </c>
+      <c r="E24" s="1">
+        <v>45829</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5">
+      <c r="B25">
+        <f>B24+1</f>
+        <v>23</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1160</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>1161</v>
+      </c>
+      <c r="E25" s="1">
+        <v>45829</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5">
+      <c r="B26">
+        <f>B25+1</f>
+        <v>24</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1163</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>1162</v>
+      </c>
+      <c r="E26" t="s">
+        <v>1117</v>
       </c>
     </row>
   </sheetData>
@@ -12047,6 +12142,10 @@
     <hyperlink ref="D20" r:id="rId18" xr:uid="{6B9F7F7E-2ABF-4562-AC3E-47C0038E2C6B}"/>
     <hyperlink ref="D21" r:id="rId19" xr:uid="{0A06A6BE-B9B1-48B2-97B6-C3461C6D5BB0}"/>
     <hyperlink ref="D22" r:id="rId20" xr:uid="{0319C961-F1BF-4356-BAFF-13C18DC5132F}"/>
+    <hyperlink ref="D23" r:id="rId21" xr:uid="{31C19267-6756-4D5D-99A0-EDB29F9E8CE1}"/>
+    <hyperlink ref="D24" r:id="rId22" xr:uid="{55AAF331-FAC5-4221-AFDB-BFD806DCF3C3}"/>
+    <hyperlink ref="D25" r:id="rId23" xr:uid="{AD7546F5-4331-49B7-823C-198D2C1D0910}"/>
+    <hyperlink ref="D26" r:id="rId24" xr:uid="{99FA9D0E-3071-4E7F-8747-B5857237671E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12979,7 +13078,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -12990,7 +13089,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>00:01</v>
+        <v>03:30</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -13189,7 +13288,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -13268,7 +13367,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -13347,7 +13446,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -13426,7 +13525,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -13505,7 +13604,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -13584,7 +13683,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -13663,7 +13762,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -13742,7 +13841,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -13821,7 +13920,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -13900,7 +13999,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -13979,7 +14078,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -14058,7 +14157,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -14137,7 +14236,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -14216,7 +14315,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -14295,7 +14394,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -14374,7 +14473,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -14453,7 +14552,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -14532,7 +14631,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -14611,7 +14710,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -14690,7 +14789,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -14769,7 +14868,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -14848,7 +14947,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -14927,7 +15026,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -15006,7 +15105,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -15085,7 +15184,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -15166,7 +15265,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -15247,7 +15346,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -15328,7 +15427,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -15407,7 +15506,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -15486,7 +15585,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -15565,7 +15664,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -15646,7 +15745,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -15727,7 +15826,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -15808,7 +15907,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -15887,7 +15986,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -15966,7 +16065,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -16045,7 +16144,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -16124,7 +16223,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -16203,7 +16302,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -16284,7 +16383,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -16365,7 +16464,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -16444,7 +16543,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -16523,7 +16622,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -16602,7 +16701,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -16681,7 +16780,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -16760,7 +16859,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -16841,7 +16940,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -16922,7 +17021,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -17001,7 +17100,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -17080,7 +17179,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -17159,7 +17258,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -17238,7 +17337,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -17317,7 +17416,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -17398,7 +17497,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -17477,7 +17576,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -17558,7 +17657,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -17637,7 +17736,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -17716,7 +17815,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -17795,7 +17894,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -17874,7 +17973,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -17953,7 +18052,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -18034,7 +18133,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -18113,7 +18212,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -18192,7 +18291,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -18274,7 +18373,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -18353,7 +18452,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -18432,7 +18531,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -18511,7 +18610,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -18590,7 +18689,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -18669,7 +18768,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -18748,7 +18847,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -18827,7 +18926,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -18906,7 +19005,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -18985,7 +19084,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -19064,7 +19163,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -19143,7 +19242,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -19222,7 +19321,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -19301,7 +19400,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -19380,7 +19479,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -19459,7 +19558,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -19538,7 +19637,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -19617,7 +19716,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -19696,7 +19795,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -19775,7 +19874,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -19854,7 +19953,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -19933,7 +20032,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -20012,7 +20111,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -20091,7 +20190,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -20170,7 +20269,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -20249,7 +20348,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -20328,7 +20427,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -20407,7 +20506,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -20486,7 +20585,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -20565,7 +20664,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -20644,7 +20743,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -20723,7 +20822,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -20802,7 +20901,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -20883,7 +20982,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -20962,7 +21061,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -21041,7 +21140,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -21120,7 +21219,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -21199,7 +21298,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -21278,7 +21377,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -21359,7 +21458,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -21440,7 +21539,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -21519,7 +21618,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -21598,7 +21697,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -21677,7 +21776,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -21756,7 +21855,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -21837,7 +21936,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -21916,7 +22015,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -21995,7 +22094,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -22074,7 +22173,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -22153,7 +22252,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -22232,7 +22331,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -22311,7 +22410,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -22390,7 +22489,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -22469,7 +22568,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -22548,7 +22647,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -22627,7 +22726,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -22706,7 +22805,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -22787,7 +22886,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -22868,7 +22967,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -22947,7 +23046,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -23026,7 +23125,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -23105,7 +23204,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -23184,7 +23283,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -23263,7 +23362,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -23345,7 +23444,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -23424,7 +23523,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -23503,7 +23602,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -23582,7 +23681,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -23661,7 +23760,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -23742,7 +23841,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -23823,7 +23922,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -23902,7 +24001,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -23981,7 +24080,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -24060,7 +24159,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -24139,7 +24238,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -24218,7 +24317,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -24297,7 +24396,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -24376,7 +24475,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -24455,7 +24554,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -24534,7 +24633,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -24613,7 +24712,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -24694,7 +24793,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -24773,7 +24872,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -24852,7 +24951,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -24931,7 +25030,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -25010,7 +25109,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -25089,7 +25188,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -25168,7 +25267,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -25247,7 +25346,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -25326,7 +25425,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -25405,7 +25504,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -25484,7 +25583,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -25563,7 +25662,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -25642,7 +25741,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -25721,7 +25820,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -25800,7 +25899,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -25879,7 +25978,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -25958,7 +26057,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -26037,7 +26136,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -26118,7 +26217,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -26197,7 +26296,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -26279,7 +26378,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -26361,7 +26460,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -26440,7 +26539,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -26519,7 +26618,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -26600,7 +26699,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -26679,7 +26778,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -26758,7 +26857,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -26837,7 +26936,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -26916,7 +27015,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -26995,7 +27094,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -27076,7 +27175,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -27155,7 +27254,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -27234,7 +27333,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -27315,7 +27414,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -27396,7 +27495,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -27477,7 +27576,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -27560,7 +27659,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -27641,7 +27740,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -27722,7 +27821,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -27803,7 +27902,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -27884,7 +27983,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -27965,7 +28064,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -28048,7 +28147,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -28131,7 +28230,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -28214,7 +28313,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -28297,7 +28396,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -28378,7 +28477,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -28459,7 +28558,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -28542,7 +28641,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -28621,7 +28720,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -28700,7 +28799,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -28779,7 +28878,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -28858,7 +28957,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -28937,7 +29036,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -29018,7 +29117,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -29097,7 +29196,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -29176,7 +29275,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -29255,7 +29354,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -29334,7 +29433,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -29413,7 +29512,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -29494,7 +29593,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -29573,7 +29672,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -29652,7 +29751,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -29733,7 +29832,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -29812,7 +29911,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -29891,7 +29990,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -29970,7 +30069,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -30049,7 +30148,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -30128,7 +30227,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -30207,7 +30306,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -30286,7 +30385,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -30365,7 +30464,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -30446,7 +30545,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -30525,7 +30624,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -30604,7 +30703,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -30683,7 +30782,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -30762,7 +30861,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -30841,7 +30940,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -30920,7 +31019,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -30999,7 +31098,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -31078,7 +31177,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -31157,7 +31256,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -31236,7 +31335,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -31315,7 +31414,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -31394,7 +31493,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -31476,7 +31575,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -31555,7 +31654,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -31634,7 +31733,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -31713,7 +31812,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -31792,7 +31891,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -31871,7 +31970,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -31950,7 +32049,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -32029,7 +32128,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -32108,7 +32207,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -32187,7 +32286,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -32266,7 +32365,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -32345,7 +32444,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -32424,7 +32523,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -32503,7 +32602,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -32582,7 +32681,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -32661,7 +32760,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -32740,7 +32839,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -32819,7 +32918,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -32898,7 +32997,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -32977,7 +33076,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -33056,7 +33155,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -33135,7 +33234,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -33214,7 +33313,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -33293,7 +33392,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -33372,7 +33471,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -33451,7 +33550,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -33530,7 +33629,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -33609,7 +33708,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -33688,7 +33787,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -33767,7 +33866,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -33846,7 +33945,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -33925,7 +34024,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -34004,7 +34103,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -34083,7 +34182,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -34162,7 +34261,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -34241,7 +34340,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -34320,7 +34419,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -34399,7 +34498,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -34478,7 +34577,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -34557,7 +34656,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -34636,7 +34735,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -34715,7 +34814,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -34794,7 +34893,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -34873,7 +34972,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -34952,7 +35051,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -35031,7 +35130,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -35110,7 +35209,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -35189,7 +35288,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -35268,7 +35367,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -35347,7 +35446,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -35426,7 +35525,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -35505,7 +35604,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -35584,7 +35683,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -35663,7 +35762,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -35742,7 +35841,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -35821,7 +35920,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -35900,7 +35999,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -35979,7 +36078,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>00:00</v>
+        <v>03:30</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>

<commit_message>
Refactor DevelopmentBadgeDashboard component to utilize useCallback for performance optimization and improve data fetching logic. Add data validation in PoliticalTrends component to handle potential format issues with mediaList and parties. Update associated Excel file to reflect recent changes.
</commit_message>
<xml_diff>
--- a/Vite-Vercel開発.xlsx
+++ b/Vite-Vercel開発.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\work-time-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAFCF071-F655-4E45-8BFA-B74FC39138C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473FC505-9E07-451D-8529-B43DDD82096A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1814" uniqueCount="1164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1831" uniqueCount="1178">
   <si>
     <t>npm install -g vercel</t>
     <phoneticPr fontId="1"/>
@@ -10928,6 +10928,80 @@
     <rPh sb="0" eb="2">
       <t>セイジ</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>選挙候補者</t>
+    <rPh sb="0" eb="2">
+      <t>センキョ</t>
+    </rPh>
+    <rPh sb="2" eb="5">
+      <t>コウホシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://work-time-tracker-5d9q.vercel.app/election-candidates</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://work-time-tracker-5d9q.vercel.app/candidate-registration</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>候補者登録</t>
+    <rPh sb="0" eb="3">
+      <t>コウホシャ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>トウロク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>カレンダー</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://work-time-tracker-5d9q.vercel.app/calendar</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://work-time-tracker-5d9q.vercel.app/admin</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>管理者ダッシュボード</t>
+    <rPh sb="0" eb="3">
+      <t>カンリシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>APIテスト</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://work-time-tracker-5d9q.vercel.app/api-test</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>開発バッジ</t>
+    <rPh sb="0" eb="2">
+      <t>カイハツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://work-time-tracker-5d9q.vercel.app/development-badges</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>プロフィール</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://work-time-tracker-5d9q.vercel.app/profile</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -11726,7 +11800,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{485A7026-3BCD-4330-8EB1-BC125AB72393}">
-  <dimension ref="B2:G26"/>
+  <dimension ref="B2:G34"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
@@ -11776,7 +11850,7 @@
     </row>
     <row r="4" spans="2:7">
       <c r="B4">
-        <f>B3+1</f>
+        <f t="shared" ref="B4:B34" si="0">B3+1</f>
         <v>2</v>
       </c>
       <c r="C4" t="s">
@@ -11791,7 +11865,7 @@
     </row>
     <row r="5" spans="2:7">
       <c r="B5">
-        <f>B4+1</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C5" t="s">
@@ -11806,7 +11880,7 @@
     </row>
     <row r="6" spans="2:7">
       <c r="B6">
-        <f>B5+1</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C6" t="s">
@@ -11821,7 +11895,7 @@
     </row>
     <row r="7" spans="2:7">
       <c r="B7">
-        <f>B6+1</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C7" t="s">
@@ -11836,7 +11910,7 @@
     </row>
     <row r="8" spans="2:7">
       <c r="B8">
-        <f>B7+1</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" t="s">
@@ -11851,7 +11925,7 @@
     </row>
     <row r="9" spans="2:7">
       <c r="B9">
-        <f>B8+1</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C9" t="s">
@@ -11866,7 +11940,7 @@
     </row>
     <row r="10" spans="2:7">
       <c r="B10">
-        <f>B9+1</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" t="s">
@@ -11881,7 +11955,7 @@
     </row>
     <row r="11" spans="2:7">
       <c r="B11">
-        <f>B10+1</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C11" t="s">
@@ -11896,7 +11970,7 @@
     </row>
     <row r="12" spans="2:7">
       <c r="B12">
-        <f>B11+1</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C12" t="s">
@@ -11911,7 +11985,7 @@
     </row>
     <row r="13" spans="2:7">
       <c r="B13">
-        <f>B12+1</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C13" t="s">
@@ -11926,7 +12000,7 @@
     </row>
     <row r="14" spans="2:7">
       <c r="B14">
-        <f>B13+1</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C14" t="s">
@@ -11941,7 +12015,7 @@
     </row>
     <row r="15" spans="2:7">
       <c r="B15">
-        <f>B14+1</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C15" t="s">
@@ -11956,7 +12030,7 @@
     </row>
     <row r="16" spans="2:7">
       <c r="B16">
-        <f>B15+1</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" t="s">
@@ -11971,7 +12045,7 @@
     </row>
     <row r="17" spans="2:5">
       <c r="B17">
-        <f>B16+1</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C17" t="s">
@@ -11986,7 +12060,7 @@
     </row>
     <row r="18" spans="2:5">
       <c r="B18">
-        <f>B17+1</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C18" t="s">
@@ -12001,7 +12075,7 @@
     </row>
     <row r="19" spans="2:5">
       <c r="B19">
-        <f>B18+1</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C19" t="s">
@@ -12016,7 +12090,7 @@
     </row>
     <row r="20" spans="2:5">
       <c r="B20">
-        <f>B19+1</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C20" t="s">
@@ -12031,7 +12105,7 @@
     </row>
     <row r="21" spans="2:5">
       <c r="B21">
-        <f>B20+1</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C21" t="s">
@@ -12046,7 +12120,7 @@
     </row>
     <row r="22" spans="2:5">
       <c r="B22">
-        <f>B21+1</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C22" t="s">
@@ -12061,7 +12135,7 @@
     </row>
     <row r="23" spans="2:5">
       <c r="B23">
-        <f>B22+1</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C23" t="s">
@@ -12076,7 +12150,7 @@
     </row>
     <row r="24" spans="2:5">
       <c r="B24">
-        <f>B23+1</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C24" t="s">
@@ -12091,7 +12165,7 @@
     </row>
     <row r="25" spans="2:5">
       <c r="B25">
-        <f>B24+1</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C25" t="s">
@@ -12106,7 +12180,7 @@
     </row>
     <row r="26" spans="2:5">
       <c r="B26">
-        <f>B25+1</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C26" t="s">
@@ -12117,6 +12191,117 @@
       </c>
       <c r="E26" t="s">
         <v>1117</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5">
+      <c r="B27">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1164</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>1165</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>1117</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5">
+      <c r="B28">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1167</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>1166</v>
+      </c>
+      <c r="E28" t="s">
+        <v>1117</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5">
+      <c r="B29">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1168</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>1169</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>1117</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5">
+      <c r="B30">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1171</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>1170</v>
+      </c>
+      <c r="E30" s="1">
+        <v>45829</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5">
+      <c r="B31">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1172</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E31" s="1">
+        <v>45829</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5">
+      <c r="B32">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1174</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>1175</v>
+      </c>
+      <c r="E32" s="1">
+        <v>45829</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5">
+      <c r="B33">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1176</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>1177</v>
+      </c>
+      <c r="E33" s="1">
+        <v>45829</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5">
+      <c r="B34">
+        <f t="shared" si="0"/>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -12146,6 +12331,13 @@
     <hyperlink ref="D24" r:id="rId22" xr:uid="{55AAF331-FAC5-4221-AFDB-BFD806DCF3C3}"/>
     <hyperlink ref="D25" r:id="rId23" xr:uid="{AD7546F5-4331-49B7-823C-198D2C1D0910}"/>
     <hyperlink ref="D26" r:id="rId24" xr:uid="{99FA9D0E-3071-4E7F-8747-B5857237671E}"/>
+    <hyperlink ref="D27" r:id="rId25" xr:uid="{33B80923-8356-43BB-A085-13ADE274A505}"/>
+    <hyperlink ref="D28" r:id="rId26" xr:uid="{5F3B3DB5-763C-4022-8575-707C6CCC2585}"/>
+    <hyperlink ref="D29" r:id="rId27" xr:uid="{ADDDDAC3-7B7B-4C47-B08A-6846C89CF20A}"/>
+    <hyperlink ref="D30" r:id="rId28" xr:uid="{4CC1F8D3-63E1-4138-9C5D-67AB034516E9}"/>
+    <hyperlink ref="D31" r:id="rId29" xr:uid="{01812CCE-47F4-4F99-B909-44E5FCCB89F6}"/>
+    <hyperlink ref="D32" r:id="rId30" xr:uid="{173501B2-7C53-49DF-A8F5-4E44C6682FBC}"/>
+    <hyperlink ref="D33" r:id="rId31" xr:uid="{82721634-7CAA-4F81-ADBC-0278598018D7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13078,7 +13270,7 @@
       MOD(NOW(),1),
       TIME(0,5,0)
     ),"HH:mm")</f>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="1">
@@ -13089,7 +13281,7 @@
     <row r="3" spans="1:65">
       <c r="A3" s="19" t="str">
         <f ca="1">TEXT(NOW(),"HH:mm")</f>
-        <v>03:30</v>
+        <v>13:17</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="17" t="s">
@@ -13288,7 +13480,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" ref="B4:B67" si="1">TEXT($C4, "HH:mm")</f>
@@ -13367,7 +13559,7 @@
     <row r="5" spans="1:65">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="1"/>
@@ -13446,7 +13638,7 @@
     <row r="6" spans="1:65">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="1"/>
@@ -13525,7 +13717,7 @@
     <row r="7" spans="1:65">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="1"/>
@@ -13604,7 +13796,7 @@
     <row r="8" spans="1:65">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="1"/>
@@ -13683,7 +13875,7 @@
     <row r="9" spans="1:65">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="1"/>
@@ -13762,7 +13954,7 @@
     <row r="10" spans="1:65">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="1"/>
@@ -13841,7 +14033,7 @@
     <row r="11" spans="1:65">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="1"/>
@@ -13920,7 +14112,7 @@
     <row r="12" spans="1:65">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="1"/>
@@ -13999,7 +14191,7 @@
     <row r="13" spans="1:65">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="1"/>
@@ -14078,7 +14270,7 @@
     <row r="14" spans="1:65">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="1"/>
@@ -14157,7 +14349,7 @@
     <row r="15" spans="1:65">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="1"/>
@@ -14236,7 +14428,7 @@
     <row r="16" spans="1:65">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="1"/>
@@ -14315,7 +14507,7 @@
     <row r="17" spans="1:65">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="1"/>
@@ -14394,7 +14586,7 @@
     <row r="18" spans="1:65">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="1"/>
@@ -14473,7 +14665,7 @@
     <row r="19" spans="1:65">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="1"/>
@@ -14552,7 +14744,7 @@
     <row r="20" spans="1:65">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="1"/>
@@ -14631,7 +14823,7 @@
     <row r="21" spans="1:65">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="1"/>
@@ -14710,7 +14902,7 @@
     <row r="22" spans="1:65">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="1"/>
@@ -14789,7 +14981,7 @@
     <row r="23" spans="1:65">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="1"/>
@@ -14868,7 +15060,7 @@
     <row r="24" spans="1:65">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="1"/>
@@ -14947,7 +15139,7 @@
     <row r="25" spans="1:65">
       <c r="A25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="1"/>
@@ -15026,7 +15218,7 @@
     <row r="26" spans="1:65">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="1"/>
@@ -15105,7 +15297,7 @@
     <row r="27" spans="1:65">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="1"/>
@@ -15184,7 +15376,7 @@
     <row r="28" spans="1:65">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="1"/>
@@ -15265,7 +15457,7 @@
     <row r="29" spans="1:65">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="1"/>
@@ -15346,7 +15538,7 @@
     <row r="30" spans="1:65">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="1"/>
@@ -15427,7 +15619,7 @@
     <row r="31" spans="1:65">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="1"/>
@@ -15506,7 +15698,7 @@
     <row r="32" spans="1:65">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="1"/>
@@ -15585,7 +15777,7 @@
     <row r="33" spans="1:65">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="1"/>
@@ -15664,7 +15856,7 @@
     <row r="34" spans="1:65">
       <c r="A34" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="1"/>
@@ -15745,7 +15937,7 @@
     <row r="35" spans="1:65">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="1"/>
@@ -15826,7 +16018,7 @@
     <row r="36" spans="1:65">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="1"/>
@@ -15907,7 +16099,7 @@
     <row r="37" spans="1:65">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="1"/>
@@ -15986,7 +16178,7 @@
     <row r="38" spans="1:65">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="1"/>
@@ -16065,7 +16257,7 @@
     <row r="39" spans="1:65">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="1"/>
@@ -16144,7 +16336,7 @@
     <row r="40" spans="1:65">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="1"/>
@@ -16223,7 +16415,7 @@
     <row r="41" spans="1:65">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="1"/>
@@ -16302,7 +16494,7 @@
     <row r="42" spans="1:65">
       <c r="A42" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="1"/>
@@ -16383,7 +16575,7 @@
     <row r="43" spans="1:65">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="1"/>
@@ -16464,7 +16656,7 @@
     <row r="44" spans="1:65">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="1"/>
@@ -16543,7 +16735,7 @@
     <row r="45" spans="1:65">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="1"/>
@@ -16622,7 +16814,7 @@
     <row r="46" spans="1:65">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="1"/>
@@ -16701,7 +16893,7 @@
     <row r="47" spans="1:65">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="1"/>
@@ -16780,7 +16972,7 @@
     <row r="48" spans="1:65">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="1"/>
@@ -16859,7 +17051,7 @@
     <row r="49" spans="1:65">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="1"/>
@@ -16940,7 +17132,7 @@
     <row r="50" spans="1:65">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="1"/>
@@ -17021,7 +17213,7 @@
     <row r="51" spans="1:65">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="1"/>
@@ -17100,7 +17292,7 @@
     <row r="52" spans="1:65">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="1"/>
@@ -17179,7 +17371,7 @@
     <row r="53" spans="1:65">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="1"/>
@@ -17258,7 +17450,7 @@
     <row r="54" spans="1:65">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="1"/>
@@ -17337,7 +17529,7 @@
     <row r="55" spans="1:65">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="1"/>
@@ -17416,7 +17608,7 @@
     <row r="56" spans="1:65">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="1"/>
@@ -17497,7 +17689,7 @@
     <row r="57" spans="1:65">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="1"/>
@@ -17576,7 +17768,7 @@
     <row r="58" spans="1:65">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="1"/>
@@ -17657,7 +17849,7 @@
     <row r="59" spans="1:65">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="1"/>
@@ -17736,7 +17928,7 @@
     <row r="60" spans="1:65">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="1"/>
@@ -17815,7 +18007,7 @@
     <row r="61" spans="1:65">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="1"/>
@@ -17894,7 +18086,7 @@
     <row r="62" spans="1:65">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="1"/>
@@ -17973,7 +18165,7 @@
     <row r="63" spans="1:65">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="1"/>
@@ -18052,7 +18244,7 @@
     <row r="64" spans="1:65">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="1"/>
@@ -18133,7 +18325,7 @@
     <row r="65" spans="1:65">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="1"/>
@@ -18212,7 +18404,7 @@
     <row r="66" spans="1:65">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" si="1"/>
@@ -18291,7 +18483,7 @@
     <row r="67" spans="1:65">
       <c r="A67" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="1"/>
@@ -18373,7 +18565,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" ref="B68:B131" si="3">TEXT($C68, "HH:mm")</f>
@@ -18452,7 +18644,7 @@
     <row r="69" spans="1:65">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="3"/>
@@ -18531,7 +18723,7 @@
     <row r="70" spans="1:65">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="3"/>
@@ -18610,7 +18802,7 @@
     <row r="71" spans="1:65">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="3"/>
@@ -18689,7 +18881,7 @@
     <row r="72" spans="1:65">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="3"/>
@@ -18768,7 +18960,7 @@
     <row r="73" spans="1:65">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="3"/>
@@ -18847,7 +19039,7 @@
     <row r="74" spans="1:65">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="3"/>
@@ -18926,7 +19118,7 @@
     <row r="75" spans="1:65">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="3"/>
@@ -19005,7 +19197,7 @@
     <row r="76" spans="1:65">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="3"/>
@@ -19084,7 +19276,7 @@
     <row r="77" spans="1:65">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="3"/>
@@ -19163,7 +19355,7 @@
     <row r="78" spans="1:65">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="3"/>
@@ -19242,7 +19434,7 @@
     <row r="79" spans="1:65">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B79" t="str">
         <f t="shared" si="3"/>
@@ -19321,7 +19513,7 @@
     <row r="80" spans="1:65">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B80" t="str">
         <f t="shared" si="3"/>
@@ -19400,7 +19592,7 @@
     <row r="81" spans="1:65">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B81" t="str">
         <f t="shared" si="3"/>
@@ -19479,7 +19671,7 @@
     <row r="82" spans="1:65">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B82" t="str">
         <f t="shared" si="3"/>
@@ -19558,7 +19750,7 @@
     <row r="83" spans="1:65">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B83" t="str">
         <f t="shared" si="3"/>
@@ -19637,7 +19829,7 @@
     <row r="84" spans="1:65">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B84" t="str">
         <f t="shared" si="3"/>
@@ -19716,7 +19908,7 @@
     <row r="85" spans="1:65">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B85" t="str">
         <f t="shared" si="3"/>
@@ -19795,7 +19987,7 @@
     <row r="86" spans="1:65">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B86" t="str">
         <f t="shared" si="3"/>
@@ -19874,7 +20066,7 @@
     <row r="87" spans="1:65">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B87" t="str">
         <f t="shared" si="3"/>
@@ -19953,7 +20145,7 @@
     <row r="88" spans="1:65">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B88" t="str">
         <f t="shared" si="3"/>
@@ -20032,7 +20224,7 @@
     <row r="89" spans="1:65">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B89" t="str">
         <f t="shared" si="3"/>
@@ -20111,7 +20303,7 @@
     <row r="90" spans="1:65">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B90" t="str">
         <f t="shared" si="3"/>
@@ -20190,7 +20382,7 @@
     <row r="91" spans="1:65">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B91" t="str">
         <f t="shared" si="3"/>
@@ -20269,7 +20461,7 @@
     <row r="92" spans="1:65">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B92" t="str">
         <f t="shared" si="3"/>
@@ -20348,7 +20540,7 @@
     <row r="93" spans="1:65">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B93" t="str">
         <f t="shared" si="3"/>
@@ -20427,7 +20619,7 @@
     <row r="94" spans="1:65">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B94" t="str">
         <f t="shared" si="3"/>
@@ -20506,7 +20698,7 @@
     <row r="95" spans="1:65">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B95" t="str">
         <f t="shared" si="3"/>
@@ -20585,7 +20777,7 @@
     <row r="96" spans="1:65">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B96" t="str">
         <f t="shared" si="3"/>
@@ -20664,7 +20856,7 @@
     <row r="97" spans="1:65">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B97" t="str">
         <f t="shared" si="3"/>
@@ -20743,7 +20935,7 @@
     <row r="98" spans="1:65">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B98" t="str">
         <f t="shared" si="3"/>
@@ -20822,7 +21014,7 @@
     <row r="99" spans="1:65">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B99" t="str">
         <f t="shared" si="3"/>
@@ -20901,7 +21093,7 @@
     <row r="100" spans="1:65">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B100" t="str">
         <f t="shared" si="3"/>
@@ -20982,7 +21174,7 @@
     <row r="101" spans="1:65">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B101" t="str">
         <f t="shared" si="3"/>
@@ -21061,7 +21253,7 @@
     <row r="102" spans="1:65">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B102" t="str">
         <f t="shared" si="3"/>
@@ -21140,7 +21332,7 @@
     <row r="103" spans="1:65">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B103" t="str">
         <f t="shared" si="3"/>
@@ -21219,7 +21411,7 @@
     <row r="104" spans="1:65">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B104" t="str">
         <f t="shared" si="3"/>
@@ -21298,7 +21490,7 @@
     <row r="105" spans="1:65">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B105" t="str">
         <f t="shared" si="3"/>
@@ -21377,7 +21569,7 @@
     <row r="106" spans="1:65">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B106" t="str">
         <f t="shared" si="3"/>
@@ -21458,7 +21650,7 @@
     <row r="107" spans="1:65">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B107" t="str">
         <f t="shared" si="3"/>
@@ -21539,7 +21731,7 @@
     <row r="108" spans="1:65">
       <c r="A108" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B108" t="str">
         <f t="shared" si="3"/>
@@ -21618,7 +21810,7 @@
     <row r="109" spans="1:65">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B109" t="str">
         <f t="shared" si="3"/>
@@ -21697,7 +21889,7 @@
     <row r="110" spans="1:65">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B110" t="str">
         <f t="shared" si="3"/>
@@ -21776,7 +21968,7 @@
     <row r="111" spans="1:65">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B111" t="str">
         <f t="shared" si="3"/>
@@ -21855,7 +22047,7 @@
     <row r="112" spans="1:65">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B112" t="str">
         <f t="shared" si="3"/>
@@ -21936,7 +22128,7 @@
     <row r="113" spans="1:65">
       <c r="A113" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B113" t="str">
         <f t="shared" si="3"/>
@@ -22015,7 +22207,7 @@
     <row r="114" spans="1:65">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B114" t="str">
         <f t="shared" si="3"/>
@@ -22094,7 +22286,7 @@
     <row r="115" spans="1:65">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B115" t="str">
         <f t="shared" si="3"/>
@@ -22173,7 +22365,7 @@
     <row r="116" spans="1:65">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B116" t="str">
         <f t="shared" si="3"/>
@@ -22252,7 +22444,7 @@
     <row r="117" spans="1:65">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B117" t="str">
         <f t="shared" si="3"/>
@@ -22331,7 +22523,7 @@
     <row r="118" spans="1:65">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B118" t="str">
         <f t="shared" si="3"/>
@@ -22410,7 +22602,7 @@
     <row r="119" spans="1:65">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B119" t="str">
         <f t="shared" si="3"/>
@@ -22489,7 +22681,7 @@
     <row r="120" spans="1:65">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B120" t="str">
         <f t="shared" si="3"/>
@@ -22568,7 +22760,7 @@
     <row r="121" spans="1:65">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="3"/>
@@ -22647,7 +22839,7 @@
     <row r="122" spans="1:65">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="3"/>
@@ -22726,7 +22918,7 @@
     <row r="123" spans="1:65">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="3"/>
@@ -22805,7 +22997,7 @@
     <row r="124" spans="1:65">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="3"/>
@@ -22886,7 +23078,7 @@
     <row r="125" spans="1:65">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="3"/>
@@ -22967,7 +23159,7 @@
     <row r="126" spans="1:65">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="3"/>
@@ -23046,7 +23238,7 @@
     <row r="127" spans="1:65">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="3"/>
@@ -23125,7 +23317,7 @@
     <row r="128" spans="1:65">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="3"/>
@@ -23204,7 +23396,7 @@
     <row r="129" spans="1:65">
       <c r="A129" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="3"/>
@@ -23283,7 +23475,7 @@
     <row r="130" spans="1:65">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="3"/>
@@ -23362,7 +23554,7 @@
     <row r="131" spans="1:65">
       <c r="A131" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B131" t="str">
         <f t="shared" si="3"/>
@@ -23444,7 +23636,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B132" t="str">
         <f t="shared" ref="B132:B168" si="5">TEXT($C132, "HH:mm")</f>
@@ -23523,7 +23715,7 @@
     <row r="133" spans="1:65">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B133" t="str">
         <f t="shared" si="5"/>
@@ -23602,7 +23794,7 @@
     <row r="134" spans="1:65">
       <c r="A134" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B134" t="str">
         <f t="shared" si="5"/>
@@ -23681,7 +23873,7 @@
     <row r="135" spans="1:65">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B135" t="str">
         <f t="shared" si="5"/>
@@ -23760,7 +23952,7 @@
     <row r="136" spans="1:65">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B136" t="str">
         <f t="shared" si="5"/>
@@ -23841,7 +24033,7 @@
     <row r="137" spans="1:65">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B137" t="str">
         <f t="shared" si="5"/>
@@ -23922,7 +24114,7 @@
     <row r="138" spans="1:65">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B138" t="str">
         <f t="shared" si="5"/>
@@ -24001,7 +24193,7 @@
     <row r="139" spans="1:65">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B139" t="str">
         <f t="shared" si="5"/>
@@ -24080,7 +24272,7 @@
     <row r="140" spans="1:65">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B140" t="str">
         <f t="shared" si="5"/>
@@ -24159,7 +24351,7 @@
     <row r="141" spans="1:65">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B141" t="str">
         <f t="shared" si="5"/>
@@ -24238,7 +24430,7 @@
     <row r="142" spans="1:65">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B142" t="str">
         <f t="shared" si="5"/>
@@ -24317,7 +24509,7 @@
     <row r="143" spans="1:65">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B143" t="str">
         <f t="shared" si="5"/>
@@ -24396,7 +24588,7 @@
     <row r="144" spans="1:65">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B144" t="str">
         <f t="shared" si="5"/>
@@ -24475,7 +24667,7 @@
     <row r="145" spans="1:65">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B145" t="str">
         <f t="shared" si="5"/>
@@ -24554,7 +24746,7 @@
     <row r="146" spans="1:65">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B146" t="str">
         <f t="shared" si="5"/>
@@ -24633,7 +24825,7 @@
     <row r="147" spans="1:65">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B147" t="str">
         <f t="shared" si="5"/>
@@ -24712,7 +24904,7 @@
     <row r="148" spans="1:65">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B148" t="str">
         <f t="shared" si="5"/>
@@ -24793,7 +24985,7 @@
     <row r="149" spans="1:65">
       <c r="A149" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B149" t="str">
         <f t="shared" si="5"/>
@@ -24872,7 +25064,7 @@
     <row r="150" spans="1:65">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B150" t="str">
         <f t="shared" si="5"/>
@@ -24951,7 +25143,7 @@
     <row r="151" spans="1:65">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B151" t="str">
         <f t="shared" si="5"/>
@@ -25030,7 +25222,7 @@
     <row r="152" spans="1:65">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B152" t="str">
         <f t="shared" si="5"/>
@@ -25109,7 +25301,7 @@
     <row r="153" spans="1:65">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B153" t="str">
         <f t="shared" si="5"/>
@@ -25188,7 +25380,7 @@
     <row r="154" spans="1:65">
       <c r="A154" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B154" t="str">
         <f t="shared" si="5"/>
@@ -25267,7 +25459,7 @@
     <row r="155" spans="1:65">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B155" t="str">
         <f t="shared" si="5"/>
@@ -25346,7 +25538,7 @@
     <row r="156" spans="1:65">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B156" t="str">
         <f t="shared" si="5"/>
@@ -25425,7 +25617,7 @@
     <row r="157" spans="1:65">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B157" t="str">
         <f t="shared" si="5"/>
@@ -25504,7 +25696,7 @@
     <row r="158" spans="1:65">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B158" t="str">
         <f t="shared" si="5"/>
@@ -25583,7 +25775,7 @@
     <row r="159" spans="1:65">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B159" t="str">
         <f t="shared" si="5"/>
@@ -25662,7 +25854,7 @@
     <row r="160" spans="1:65">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B160" t="str">
         <f t="shared" si="5"/>
@@ -25741,7 +25933,7 @@
     <row r="161" spans="1:65">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B161" t="str">
         <f t="shared" si="5"/>
@@ -25820,7 +26012,7 @@
     <row r="162" spans="1:65">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B162" t="str">
         <f t="shared" si="5"/>
@@ -25899,7 +26091,7 @@
     <row r="163" spans="1:65">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B163" t="str">
         <f t="shared" si="5"/>
@@ -25978,7 +26170,7 @@
     <row r="164" spans="1:65">
       <c r="A164" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B164" t="str">
         <f t="shared" si="5"/>
@@ -26057,7 +26249,7 @@
     <row r="165" spans="1:65">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B165" t="str">
         <f t="shared" si="5"/>
@@ -26136,7 +26328,7 @@
     <row r="166" spans="1:65">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B166" t="str">
         <f t="shared" si="5"/>
@@ -26217,7 +26409,7 @@
     <row r="167" spans="1:65">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B167" t="str">
         <f t="shared" si="5"/>
@@ -26296,7 +26488,7 @@
     <row r="168" spans="1:65">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B168" t="str">
         <f t="shared" si="5"/>
@@ -26378,7 +26570,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B169" t="str">
         <f>TEXT($C169, "HH:mm")</f>
@@ -26460,7 +26652,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B170" t="str">
         <f t="shared" ref="B170:B233" si="7">TEXT($C170, "HH:mm")</f>
@@ -26539,7 +26731,7 @@
     <row r="171" spans="1:65">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B171" t="str">
         <f t="shared" si="7"/>
@@ -26618,7 +26810,7 @@
     <row r="172" spans="1:65">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B172" t="str">
         <f t="shared" si="7"/>
@@ -26699,7 +26891,7 @@
     <row r="173" spans="1:65">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B173" t="str">
         <f t="shared" si="7"/>
@@ -26778,7 +26970,7 @@
     <row r="174" spans="1:65">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B174" t="str">
         <f t="shared" si="7"/>
@@ -26857,7 +27049,7 @@
     <row r="175" spans="1:65">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B175" t="str">
         <f t="shared" si="7"/>
@@ -26936,7 +27128,7 @@
     <row r="176" spans="1:65">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B176" t="str">
         <f t="shared" si="7"/>
@@ -27015,7 +27207,7 @@
     <row r="177" spans="1:65">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B177" t="str">
         <f t="shared" si="7"/>
@@ -27094,7 +27286,7 @@
     <row r="178" spans="1:65">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B178" t="str">
         <f t="shared" si="7"/>
@@ -27175,7 +27367,7 @@
     <row r="179" spans="1:65">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B179" t="str">
         <f t="shared" si="7"/>
@@ -27254,7 +27446,7 @@
     <row r="180" spans="1:65">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B180" t="str">
         <f t="shared" si="7"/>
@@ -27333,7 +27525,7 @@
     <row r="181" spans="1:65">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B181" t="str">
         <f t="shared" si="7"/>
@@ -27414,7 +27606,7 @@
     <row r="182" spans="1:65">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B182" t="str">
         <f t="shared" si="7"/>
@@ -27495,7 +27687,7 @@
     <row r="183" spans="1:65">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B183" t="str">
         <f t="shared" si="7"/>
@@ -27576,7 +27768,7 @@
     <row r="184" spans="1:65">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B184" t="str">
         <f t="shared" si="7"/>
@@ -27659,7 +27851,7 @@
     <row r="185" spans="1:65">
       <c r="A185" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B185" t="str">
         <f t="shared" si="7"/>
@@ -27740,7 +27932,7 @@
     <row r="186" spans="1:65">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B186" t="str">
         <f t="shared" si="7"/>
@@ -27821,7 +28013,7 @@
     <row r="187" spans="1:65">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B187" t="str">
         <f t="shared" si="7"/>
@@ -27902,7 +28094,7 @@
     <row r="188" spans="1:65">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B188" t="str">
         <f t="shared" si="7"/>
@@ -27983,7 +28175,7 @@
     <row r="189" spans="1:65">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B189" t="str">
         <f t="shared" si="7"/>
@@ -28064,7 +28256,7 @@
     <row r="190" spans="1:65">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B190" t="str">
         <f t="shared" si="7"/>
@@ -28147,7 +28339,7 @@
     <row r="191" spans="1:65">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B191" t="str">
         <f t="shared" si="7"/>
@@ -28230,7 +28422,7 @@
     <row r="192" spans="1:65">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B192" t="str">
         <f t="shared" si="7"/>
@@ -28313,7 +28505,7 @@
     <row r="193" spans="1:65">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B193" t="str">
         <f t="shared" si="7"/>
@@ -28396,7 +28588,7 @@
     <row r="194" spans="1:65">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B194" t="str">
         <f t="shared" si="7"/>
@@ -28477,7 +28669,7 @@
     <row r="195" spans="1:65">
       <c r="A195" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B195" t="str">
         <f t="shared" si="7"/>
@@ -28558,7 +28750,7 @@
     <row r="196" spans="1:65">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B196" t="str">
         <f t="shared" si="7"/>
@@ -28641,7 +28833,7 @@
     <row r="197" spans="1:65">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B197" t="str">
         <f t="shared" si="7"/>
@@ -28720,7 +28912,7 @@
     <row r="198" spans="1:65">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B198" t="str">
         <f t="shared" si="7"/>
@@ -28799,7 +28991,7 @@
     <row r="199" spans="1:65">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B199" t="str">
         <f t="shared" si="7"/>
@@ -28878,7 +29070,7 @@
     <row r="200" spans="1:65">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B200" t="str">
         <f t="shared" si="7"/>
@@ -28957,7 +29149,7 @@
     <row r="201" spans="1:65">
       <c r="A201" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B201" t="str">
         <f t="shared" si="7"/>
@@ -29036,7 +29228,7 @@
     <row r="202" spans="1:65">
       <c r="A202" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B202" t="str">
         <f t="shared" si="7"/>
@@ -29117,7 +29309,7 @@
     <row r="203" spans="1:65">
       <c r="A203" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B203" t="str">
         <f t="shared" si="7"/>
@@ -29196,7 +29388,7 @@
     <row r="204" spans="1:65">
       <c r="A204" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B204" t="str">
         <f t="shared" si="7"/>
@@ -29275,7 +29467,7 @@
     <row r="205" spans="1:65">
       <c r="A205" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B205" t="str">
         <f t="shared" si="7"/>
@@ -29354,7 +29546,7 @@
     <row r="206" spans="1:65">
       <c r="A206" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B206" t="str">
         <f t="shared" si="7"/>
@@ -29433,7 +29625,7 @@
     <row r="207" spans="1:65">
       <c r="A207" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B207" t="str">
         <f t="shared" si="7"/>
@@ -29512,7 +29704,7 @@
     <row r="208" spans="1:65">
       <c r="A208" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B208" t="str">
         <f t="shared" si="7"/>
@@ -29593,7 +29785,7 @@
     <row r="209" spans="1:65">
       <c r="A209" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B209" t="str">
         <f t="shared" si="7"/>
@@ -29672,7 +29864,7 @@
     <row r="210" spans="1:65">
       <c r="A210" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B210" t="str">
         <f t="shared" si="7"/>
@@ -29751,7 +29943,7 @@
     <row r="211" spans="1:65">
       <c r="A211" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B211" t="str">
         <f t="shared" si="7"/>
@@ -29832,7 +30024,7 @@
     <row r="212" spans="1:65">
       <c r="A212" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B212" t="str">
         <f t="shared" si="7"/>
@@ -29911,7 +30103,7 @@
     <row r="213" spans="1:65">
       <c r="A213" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B213" t="str">
         <f t="shared" si="7"/>
@@ -29990,7 +30182,7 @@
     <row r="214" spans="1:65">
       <c r="A214" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B214" t="str">
         <f t="shared" si="7"/>
@@ -30069,7 +30261,7 @@
     <row r="215" spans="1:65">
       <c r="A215" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B215" t="str">
         <f t="shared" si="7"/>
@@ -30148,7 +30340,7 @@
     <row r="216" spans="1:65">
       <c r="A216" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B216" t="str">
         <f t="shared" si="7"/>
@@ -30227,7 +30419,7 @@
     <row r="217" spans="1:65">
       <c r="A217" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B217" t="str">
         <f t="shared" si="7"/>
@@ -30306,7 +30498,7 @@
     <row r="218" spans="1:65">
       <c r="A218" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B218" t="str">
         <f t="shared" si="7"/>
@@ -30385,7 +30577,7 @@
     <row r="219" spans="1:65">
       <c r="A219" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B219" t="str">
         <f t="shared" si="7"/>
@@ -30464,7 +30656,7 @@
     <row r="220" spans="1:65">
       <c r="A220" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B220" t="str">
         <f t="shared" si="7"/>
@@ -30545,7 +30737,7 @@
     <row r="221" spans="1:65">
       <c r="A221" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B221" t="str">
         <f t="shared" si="7"/>
@@ -30624,7 +30816,7 @@
     <row r="222" spans="1:65">
       <c r="A222" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B222" t="str">
         <f t="shared" si="7"/>
@@ -30703,7 +30895,7 @@
     <row r="223" spans="1:65">
       <c r="A223" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B223" t="str">
         <f t="shared" si="7"/>
@@ -30782,7 +30974,7 @@
     <row r="224" spans="1:65">
       <c r="A224" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B224" t="str">
         <f t="shared" si="7"/>
@@ -30861,7 +31053,7 @@
     <row r="225" spans="1:65">
       <c r="A225" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B225" t="str">
         <f t="shared" si="7"/>
@@ -30940,7 +31132,7 @@
     <row r="226" spans="1:65">
       <c r="A226" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B226" t="str">
         <f t="shared" si="7"/>
@@ -31019,7 +31211,7 @@
     <row r="227" spans="1:65">
       <c r="A227" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B227" t="str">
         <f t="shared" si="7"/>
@@ -31098,7 +31290,7 @@
     <row r="228" spans="1:65">
       <c r="A228" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B228" t="str">
         <f t="shared" si="7"/>
@@ -31177,7 +31369,7 @@
     <row r="229" spans="1:65">
       <c r="A229" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B229" t="str">
         <f t="shared" si="7"/>
@@ -31256,7 +31448,7 @@
     <row r="230" spans="1:65">
       <c r="A230" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B230" t="str">
         <f t="shared" si="7"/>
@@ -31335,7 +31527,7 @@
     <row r="231" spans="1:65">
       <c r="A231" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B231" t="str">
         <f t="shared" si="7"/>
@@ -31414,7 +31606,7 @@
     <row r="232" spans="1:65">
       <c r="A232" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B232" t="str">
         <f t="shared" si="7"/>
@@ -31493,7 +31685,7 @@
     <row r="233" spans="1:65">
       <c r="A233" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B233" t="str">
         <f t="shared" si="7"/>
@@ -31575,7 +31767,7 @@
   FLOOR( MOD(NOW(),1), TIME(0,5,0) ),
   "HH:mm"
 )</f>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B234" t="str">
         <f t="shared" ref="B234:B291" si="9">TEXT($C234, "HH:mm")</f>
@@ -31654,7 +31846,7 @@
     <row r="235" spans="1:65">
       <c r="A235" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B235" t="str">
         <f t="shared" si="9"/>
@@ -31733,7 +31925,7 @@
     <row r="236" spans="1:65">
       <c r="A236" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B236" t="str">
         <f t="shared" si="9"/>
@@ -31812,7 +32004,7 @@
     <row r="237" spans="1:65">
       <c r="A237" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B237" t="str">
         <f t="shared" si="9"/>
@@ -31891,7 +32083,7 @@
     <row r="238" spans="1:65">
       <c r="A238" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B238" t="str">
         <f t="shared" si="9"/>
@@ -31970,7 +32162,7 @@
     <row r="239" spans="1:65">
       <c r="A239" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B239" t="str">
         <f t="shared" si="9"/>
@@ -32049,7 +32241,7 @@
     <row r="240" spans="1:65">
       <c r="A240" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B240" t="str">
         <f t="shared" si="9"/>
@@ -32128,7 +32320,7 @@
     <row r="241" spans="1:65">
       <c r="A241" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B241" t="str">
         <f t="shared" si="9"/>
@@ -32207,7 +32399,7 @@
     <row r="242" spans="1:65">
       <c r="A242" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B242" t="str">
         <f t="shared" si="9"/>
@@ -32286,7 +32478,7 @@
     <row r="243" spans="1:65">
       <c r="A243" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B243" t="str">
         <f t="shared" si="9"/>
@@ -32365,7 +32557,7 @@
     <row r="244" spans="1:65">
       <c r="A244" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B244" t="str">
         <f t="shared" si="9"/>
@@ -32444,7 +32636,7 @@
     <row r="245" spans="1:65">
       <c r="A245" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B245" t="str">
         <f t="shared" si="9"/>
@@ -32523,7 +32715,7 @@
     <row r="246" spans="1:65">
       <c r="A246" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B246" t="str">
         <f t="shared" si="9"/>
@@ -32602,7 +32794,7 @@
     <row r="247" spans="1:65">
       <c r="A247" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B247" t="str">
         <f t="shared" si="9"/>
@@ -32681,7 +32873,7 @@
     <row r="248" spans="1:65">
       <c r="A248" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B248" t="str">
         <f t="shared" si="9"/>
@@ -32760,7 +32952,7 @@
     <row r="249" spans="1:65">
       <c r="A249" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B249" t="str">
         <f t="shared" si="9"/>
@@ -32839,7 +33031,7 @@
     <row r="250" spans="1:65">
       <c r="A250" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B250" t="str">
         <f t="shared" si="9"/>
@@ -32918,7 +33110,7 @@
     <row r="251" spans="1:65">
       <c r="A251" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B251" t="str">
         <f t="shared" si="9"/>
@@ -32997,7 +33189,7 @@
     <row r="252" spans="1:65">
       <c r="A252" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B252" t="str">
         <f t="shared" si="9"/>
@@ -33076,7 +33268,7 @@
     <row r="253" spans="1:65">
       <c r="A253" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B253" t="str">
         <f t="shared" si="9"/>
@@ -33155,7 +33347,7 @@
     <row r="254" spans="1:65">
       <c r="A254" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B254" t="str">
         <f t="shared" si="9"/>
@@ -33234,7 +33426,7 @@
     <row r="255" spans="1:65">
       <c r="A255" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B255" t="str">
         <f t="shared" si="9"/>
@@ -33313,7 +33505,7 @@
     <row r="256" spans="1:65">
       <c r="A256" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B256" t="str">
         <f t="shared" si="9"/>
@@ -33392,7 +33584,7 @@
     <row r="257" spans="1:65">
       <c r="A257" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B257" t="str">
         <f t="shared" si="9"/>
@@ -33471,7 +33663,7 @@
     <row r="258" spans="1:65">
       <c r="A258" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B258" t="str">
         <f t="shared" si="9"/>
@@ -33550,7 +33742,7 @@
     <row r="259" spans="1:65">
       <c r="A259" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B259" t="str">
         <f t="shared" si="9"/>
@@ -33629,7 +33821,7 @@
     <row r="260" spans="1:65">
       <c r="A260" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B260" t="str">
         <f t="shared" si="9"/>
@@ -33708,7 +33900,7 @@
     <row r="261" spans="1:65">
       <c r="A261" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B261" t="str">
         <f t="shared" si="9"/>
@@ -33787,7 +33979,7 @@
     <row r="262" spans="1:65">
       <c r="A262" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B262" t="str">
         <f t="shared" si="9"/>
@@ -33866,7 +34058,7 @@
     <row r="263" spans="1:65">
       <c r="A263" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B263" t="str">
         <f t="shared" si="9"/>
@@ -33945,7 +34137,7 @@
     <row r="264" spans="1:65">
       <c r="A264" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B264" t="str">
         <f t="shared" si="9"/>
@@ -34024,7 +34216,7 @@
     <row r="265" spans="1:65">
       <c r="A265" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B265" t="str">
         <f t="shared" si="9"/>
@@ -34103,7 +34295,7 @@
     <row r="266" spans="1:65">
       <c r="A266" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B266" t="str">
         <f t="shared" si="9"/>
@@ -34182,7 +34374,7 @@
     <row r="267" spans="1:65">
       <c r="A267" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B267" t="str">
         <f t="shared" si="9"/>
@@ -34261,7 +34453,7 @@
     <row r="268" spans="1:65">
       <c r="A268" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B268" t="str">
         <f t="shared" si="9"/>
@@ -34340,7 +34532,7 @@
     <row r="269" spans="1:65">
       <c r="A269" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B269" t="str">
         <f t="shared" si="9"/>
@@ -34419,7 +34611,7 @@
     <row r="270" spans="1:65">
       <c r="A270" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B270" t="str">
         <f t="shared" si="9"/>
@@ -34498,7 +34690,7 @@
     <row r="271" spans="1:65">
       <c r="A271" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B271" t="str">
         <f t="shared" si="9"/>
@@ -34577,7 +34769,7 @@
     <row r="272" spans="1:65">
       <c r="A272" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B272" t="str">
         <f t="shared" si="9"/>
@@ -34656,7 +34848,7 @@
     <row r="273" spans="1:65">
       <c r="A273" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B273" t="str">
         <f t="shared" si="9"/>
@@ -34735,7 +34927,7 @@
     <row r="274" spans="1:65">
       <c r="A274" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B274" t="str">
         <f t="shared" si="9"/>
@@ -34814,7 +35006,7 @@
     <row r="275" spans="1:65">
       <c r="A275" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B275" t="str">
         <f t="shared" si="9"/>
@@ -34893,7 +35085,7 @@
     <row r="276" spans="1:65">
       <c r="A276" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B276" t="str">
         <f t="shared" si="9"/>
@@ -34972,7 +35164,7 @@
     <row r="277" spans="1:65">
       <c r="A277" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B277" t="str">
         <f t="shared" si="9"/>
@@ -35051,7 +35243,7 @@
     <row r="278" spans="1:65">
       <c r="A278" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B278" t="str">
         <f t="shared" si="9"/>
@@ -35130,7 +35322,7 @@
     <row r="279" spans="1:65">
       <c r="A279" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B279" t="str">
         <f t="shared" si="9"/>
@@ -35209,7 +35401,7 @@
     <row r="280" spans="1:65">
       <c r="A280" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B280" t="str">
         <f t="shared" si="9"/>
@@ -35288,7 +35480,7 @@
     <row r="281" spans="1:65">
       <c r="A281" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B281" t="str">
         <f t="shared" si="9"/>
@@ -35367,7 +35559,7 @@
     <row r="282" spans="1:65">
       <c r="A282" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B282" t="str">
         <f t="shared" si="9"/>
@@ -35446,7 +35638,7 @@
     <row r="283" spans="1:65">
       <c r="A283" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B283" t="str">
         <f t="shared" si="9"/>
@@ -35525,7 +35717,7 @@
     <row r="284" spans="1:65">
       <c r="A284" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B284" t="str">
         <f t="shared" si="9"/>
@@ -35604,7 +35796,7 @@
     <row r="285" spans="1:65">
       <c r="A285" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B285" t="str">
         <f t="shared" si="9"/>
@@ -35683,7 +35875,7 @@
     <row r="286" spans="1:65">
       <c r="A286" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B286" t="str">
         <f t="shared" si="9"/>
@@ -35762,7 +35954,7 @@
     <row r="287" spans="1:65">
       <c r="A287" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B287" t="str">
         <f t="shared" si="9"/>
@@ -35841,7 +36033,7 @@
     <row r="288" spans="1:65">
       <c r="A288" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B288" t="str">
         <f t="shared" si="9"/>
@@ -35920,7 +36112,7 @@
     <row r="289" spans="1:65">
       <c r="A289" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B289" t="str">
         <f t="shared" si="9"/>
@@ -35999,7 +36191,7 @@
     <row r="290" spans="1:65">
       <c r="A290" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B290" t="str">
         <f t="shared" si="9"/>
@@ -36078,7 +36270,7 @@
     <row r="291" spans="1:65">
       <c r="A291" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>03:30</v>
+        <v>13:15</v>
       </c>
       <c r="B291" t="str">
         <f t="shared" si="9"/>

</xml_diff>